<commit_message>
Update RCA model info workbook
</commit_message>
<xml_diff>
--- a/eBus_Functions/Post_Processing/Root_Cause_Analysis_Work/info/eBus_Model_Info.xlsx
+++ b/eBus_Functions/Post_Processing/Root_Cause_Analysis_Work/info/eBus_Model_Info.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TempData\Github\eBus_Tool\eBus_Functions\Post_Processing\Root_Cause_Analysis_Work\info\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF1D4BBC-584A-40CA-865B-5B6F818D26AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28078C16-08E2-4DCC-BFC2-A6EFE62C8FD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Block Diagram" sheetId="1" r:id="rId1"/>
+    <sheet name="Block_Diagram" sheetId="1" r:id="rId1"/>
     <sheet name="Signal_Evaluation" sheetId="2" r:id="rId2"/>
     <sheet name="Specifications" sheetId="3" r:id="rId3"/>
   </sheets>
@@ -1210,6 +1210,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1223,9 +1226,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1630,7 +1630,7 @@
     </row>
     <row r="29" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G29" s="6"/>
-      <c r="H29" s="36" t="s">
+      <c r="H29" s="31" t="s">
         <v>6</v>
       </c>
       <c r="I29" s="7" t="s">
@@ -1639,14 +1639,14 @@
     </row>
     <row r="30" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G30" s="8"/>
-      <c r="H30" s="31"/>
+      <c r="H30" s="32"/>
       <c r="I30" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="31" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G31" s="9"/>
-      <c r="H31" s="32"/>
+      <c r="H31" s="33"/>
       <c r="I31" s="2" t="s">
         <v>32</v>
       </c>
@@ -1655,7 +1655,7 @@
       <c r="G32" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="H32" s="33" t="s">
+      <c r="H32" s="34" t="s">
         <v>0</v>
       </c>
       <c r="I32" s="7" t="s">
@@ -1666,7 +1666,7 @@
       <c r="G33" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="H33" s="34"/>
+      <c r="H33" s="35"/>
       <c r="I33" s="1" t="s">
         <v>12</v>
       </c>
@@ -1675,35 +1675,35 @@
       <c r="G34" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="H34" s="34"/>
+      <c r="H34" s="35"/>
       <c r="I34" s="1"/>
     </row>
     <row r="35" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G35" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="H35" s="34"/>
+      <c r="H35" s="35"/>
       <c r="I35" s="1"/>
     </row>
     <row r="36" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G36" s="8" t="s">
         <v>179</v>
       </c>
-      <c r="H36" s="34"/>
+      <c r="H36" s="35"/>
       <c r="I36" s="1"/>
     </row>
     <row r="37" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G37" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="H37" s="35"/>
+      <c r="H37" s="36"/>
       <c r="I37" s="2"/>
     </row>
     <row r="38" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G38" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="H38" s="36" t="s">
+      <c r="H38" s="31" t="s">
         <v>2</v>
       </c>
       <c r="I38" s="7" t="s">
@@ -1714,7 +1714,7 @@
       <c r="G39" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="H39" s="32"/>
+      <c r="H39" s="33"/>
       <c r="I39" s="2" t="s">
         <v>172</v>
       </c>
@@ -1723,7 +1723,7 @@
       <c r="G40" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="H40" s="33" t="s">
+      <c r="H40" s="34" t="s">
         <v>106</v>
       </c>
       <c r="I40" s="7" t="s">
@@ -1734,77 +1734,77 @@
       <c r="G41" s="8" t="s">
         <v>172</v>
       </c>
-      <c r="H41" s="34"/>
+      <c r="H41" s="35"/>
       <c r="I41" s="1" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="42" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G42" s="8"/>
-      <c r="H42" s="34"/>
+      <c r="H42" s="35"/>
       <c r="I42" s="1" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="43" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G43" s="8"/>
-      <c r="H43" s="34"/>
+      <c r="H43" s="35"/>
       <c r="I43" s="1" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="44" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G44" s="8"/>
-      <c r="H44" s="34"/>
+      <c r="H44" s="35"/>
       <c r="I44" s="1" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="45" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G45" s="8"/>
-      <c r="H45" s="34"/>
+      <c r="H45" s="35"/>
       <c r="I45" s="1" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="46" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G46" s="8"/>
-      <c r="H46" s="34"/>
+      <c r="H46" s="35"/>
       <c r="I46" s="1" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="47" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G47" s="8"/>
-      <c r="H47" s="34"/>
+      <c r="H47" s="35"/>
       <c r="I47" s="1" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="48" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G48" s="8"/>
-      <c r="H48" s="34"/>
+      <c r="H48" s="35"/>
       <c r="I48" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="49" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G49" s="8"/>
-      <c r="H49" s="34"/>
+      <c r="H49" s="35"/>
       <c r="I49" s="1" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="50" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G50" s="8"/>
-      <c r="H50" s="34"/>
+      <c r="H50" s="35"/>
       <c r="I50" s="1" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="51" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G51" s="9"/>
-      <c r="H51" s="35"/>
+      <c r="H51" s="36"/>
       <c r="I51" s="2" t="s">
         <v>176</v>
       </c>
@@ -1813,7 +1813,7 @@
       <c r="G52" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="H52" s="36" t="s">
+      <c r="H52" s="31" t="s">
         <v>107</v>
       </c>
       <c r="I52" s="7" t="s">
@@ -1824,28 +1824,28 @@
       <c r="G53" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="H53" s="31"/>
+      <c r="H53" s="32"/>
       <c r="I53" s="1" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="54" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G54" s="8"/>
-      <c r="H54" s="31"/>
+      <c r="H54" s="32"/>
       <c r="I54" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="55" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G55" s="8"/>
-      <c r="H55" s="31"/>
+      <c r="H55" s="32"/>
       <c r="I55" s="1" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="56" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G56" s="8"/>
-      <c r="H56" s="31"/>
+      <c r="H56" s="32"/>
       <c r="I56" s="1" t="s">
         <v>16</v>
       </c>
@@ -1865,7 +1865,7 @@
       <c r="G58" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="H58" s="33" t="s">
+      <c r="H58" s="34" t="s">
         <v>108</v>
       </c>
       <c r="I58" s="7" t="s">
@@ -1874,7 +1874,7 @@
     </row>
     <row r="59" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G59" s="8"/>
-      <c r="H59" s="34"/>
+      <c r="H59" s="35"/>
       <c r="I59" s="1" t="s">
         <v>181</v>
       </c>
@@ -1883,7 +1883,7 @@
       <c r="G60" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="H60" s="36" t="s">
+      <c r="H60" s="31" t="s">
         <v>19</v>
       </c>
       <c r="I60" s="7" t="s">
@@ -1894,42 +1894,42 @@
       <c r="G61" s="8" t="s">
         <v>180</v>
       </c>
-      <c r="H61" s="31"/>
+      <c r="H61" s="32"/>
       <c r="I61" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="62" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G62" s="8"/>
-      <c r="H62" s="31"/>
+      <c r="H62" s="32"/>
       <c r="I62" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="63" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G63" s="8"/>
-      <c r="H63" s="31"/>
+      <c r="H63" s="32"/>
       <c r="I63" s="1" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="64" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G64" s="8"/>
-      <c r="H64" s="31"/>
+      <c r="H64" s="32"/>
       <c r="I64" s="1" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="65" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G65" s="8"/>
-      <c r="H65" s="31"/>
+      <c r="H65" s="32"/>
       <c r="I65" s="1" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="66" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G66" s="9"/>
-      <c r="H66" s="32"/>
+      <c r="H66" s="33"/>
       <c r="I66" s="2" t="s">
         <v>67</v>
       </c>
@@ -1938,7 +1938,7 @@
       <c r="G67" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="H67" s="31" t="s">
+      <c r="H67" s="32" t="s">
         <v>109</v>
       </c>
       <c r="I67" s="1" t="s">
@@ -1947,35 +1947,35 @@
     </row>
     <row r="68" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G68" s="8"/>
-      <c r="H68" s="31"/>
+      <c r="H68" s="32"/>
       <c r="I68" s="1" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="69" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G69" s="8"/>
-      <c r="H69" s="31"/>
+      <c r="H69" s="32"/>
       <c r="I69" s="1" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="70" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G70" s="8"/>
-      <c r="H70" s="31"/>
+      <c r="H70" s="32"/>
       <c r="I70" s="1" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="71" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G71" s="8"/>
-      <c r="H71" s="31"/>
+      <c r="H71" s="32"/>
       <c r="I71" s="1" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="72" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G72" s="9"/>
-      <c r="H72" s="32"/>
+      <c r="H72" s="33"/>
       <c r="I72" s="2" t="s">
         <v>77</v>
       </c>
@@ -1984,7 +1984,7 @@
       <c r="G73" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="H73" s="33" t="s">
+      <c r="H73" s="34" t="s">
         <v>110</v>
       </c>
       <c r="I73" s="7" t="s">
@@ -1995,28 +1995,28 @@
       <c r="G74" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="H74" s="34"/>
+      <c r="H74" s="35"/>
       <c r="I74" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="75" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G75" s="8"/>
-      <c r="H75" s="34"/>
+      <c r="H75" s="35"/>
       <c r="I75" s="1" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="76" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G76" s="9"/>
-      <c r="H76" s="35"/>
+      <c r="H76" s="36"/>
       <c r="I76" s="2" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="77" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G77" s="8"/>
-      <c r="H77" s="31" t="s">
+      <c r="H77" s="32" t="s">
         <v>111</v>
       </c>
       <c r="I77" s="1" t="s">
@@ -2025,30 +2025,30 @@
     </row>
     <row r="78" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G78" s="8"/>
-      <c r="H78" s="31"/>
+      <c r="H78" s="32"/>
       <c r="I78" s="1" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="79" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G79" s="9"/>
-      <c r="H79" s="32"/>
+      <c r="H79" s="33"/>
       <c r="I79" s="2" t="s">
         <v>185</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="H67:H72"/>
+    <mergeCell ref="H73:H76"/>
+    <mergeCell ref="H52:H56"/>
+    <mergeCell ref="H60:H66"/>
+    <mergeCell ref="H77:H79"/>
     <mergeCell ref="H29:H31"/>
     <mergeCell ref="H32:H37"/>
     <mergeCell ref="H38:H39"/>
     <mergeCell ref="H40:H51"/>
     <mergeCell ref="H58:H59"/>
-    <mergeCell ref="H67:H72"/>
-    <mergeCell ref="H73:H76"/>
-    <mergeCell ref="H52:H56"/>
-    <mergeCell ref="H60:H66"/>
-    <mergeCell ref="H77:H79"/>
   </mergeCells>
   <conditionalFormatting sqref="I29:I79 G29:G79">
     <cfRule type="duplicateValues" dxfId="4" priority="1"/>

</xml_diff>

<commit_message>
Use workbook time signal as RCA reference time
</commit_message>
<xml_diff>
--- a/eBus_Functions/Post_Processing/Root_Cause_Analysis_Work/info/eBus_Model_Info.xlsx
+++ b/eBus_Functions/Post_Processing/Root_Cause_Analysis_Work/info/eBus_Model_Info.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TempData\Github\eBus_Tool\eBus_Functions\Post_Processing\Root_Cause_Analysis_Work\info\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28078C16-08E2-4DCC-BFC2-A6EFE62C8FD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDB3083A-0D9A-4053-A0E4-13B87157D318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Block_Diagram" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="294">
   <si>
     <t>Driver</t>
   </si>
@@ -897,6 +897,18 @@
   </si>
   <si>
     <t>VDy_axleLoss_x_speedAxleOut_rpm</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>sec</t>
+  </si>
+  <si>
+    <t>time_sim</t>
+  </si>
+  <si>
+    <t>logout.sec</t>
   </si>
 </sst>
 </file>
@@ -2061,7 +2073,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFA16316-83DB-41C7-8B25-B191695DD108}">
-  <dimension ref="A1:L100"/>
+  <dimension ref="A1:L101"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.109375" bestFit="1" customWidth="1"/>
@@ -2105,54 +2117,51 @@
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A2" s="24" t="s">
-        <v>89</v>
+      <c r="A2" s="27" t="s">
+        <v>96</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>29</v>
+        <v>290</v>
       </c>
       <c r="C2" s="25" t="s">
-        <v>98</v>
+        <v>291</v>
       </c>
       <c r="D2" s="29" t="s">
-        <v>88</v>
+        <v>292</v>
       </c>
       <c r="E2" s="26" t="s">
-        <v>30</v>
+        <v>293</v>
       </c>
       <c r="F2" s="26" t="s">
-        <v>30</v>
+        <v>293</v>
       </c>
       <c r="G2" s="26" t="s">
-        <v>30</v>
+        <v>293</v>
       </c>
       <c r="H2" s="11"/>
       <c r="I2" s="11"/>
-      <c r="J2" s="11"/>
-      <c r="K2" s="11"/>
-      <c r="L2" s="11"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="24" t="s">
         <v>89</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="C3" s="25" t="s">
-        <v>1</v>
+        <v>98</v>
       </c>
       <c r="D3" s="29" t="s">
-        <v>188</v>
+        <v>88</v>
       </c>
       <c r="E3" s="26" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F3" s="26" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G3" s="26" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H3" s="11"/>
       <c r="I3" s="11"/>
@@ -2165,22 +2174,22 @@
         <v>89</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="C4" s="25" t="s">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="D4" s="29" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E4" s="26" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="F4" s="26" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="G4" s="26" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="H4" s="11"/>
       <c r="I4" s="11"/>
@@ -2189,26 +2198,26 @@
       <c r="L4" s="11"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A5" s="27" t="s">
-        <v>96</v>
+      <c r="A5" s="24" t="s">
+        <v>89</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="C5" s="25" t="s">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="D5" s="29" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E5" s="26" t="s">
-        <v>276</v>
+        <v>34</v>
       </c>
       <c r="F5" s="26" t="s">
-        <v>276</v>
+        <v>34</v>
       </c>
       <c r="G5" s="26" t="s">
-        <v>276</v>
+        <v>34</v>
       </c>
       <c r="H5" s="11"/>
       <c r="I5" s="11"/>
@@ -2221,22 +2230,22 @@
         <v>96</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C6" s="25" t="s">
         <v>1</v>
       </c>
       <c r="D6" s="29" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E6" s="26" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F6" s="26" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="G6" s="26" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H6" s="11"/>
       <c r="I6" s="11"/>
@@ -2245,26 +2254,26 @@
       <c r="L6" s="11"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A7" s="24" t="s">
-        <v>97</v>
+      <c r="A7" s="27" t="s">
+        <v>96</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>171</v>
+        <v>12</v>
       </c>
       <c r="C7" s="25" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D7" s="29" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E7" s="26" t="s">
-        <v>186</v>
+        <v>277</v>
       </c>
       <c r="F7" s="26" t="s">
-        <v>186</v>
+        <v>277</v>
       </c>
       <c r="G7" s="26" t="s">
-        <v>186</v>
+        <v>277</v>
       </c>
       <c r="H7" s="11"/>
       <c r="I7" s="11"/>
@@ -2277,13 +2286,13 @@
         <v>97</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C8" s="25" t="s">
         <v>3</v>
       </c>
       <c r="D8" s="29" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E8" s="26" t="s">
         <v>186</v>
@@ -2301,26 +2310,26 @@
       <c r="L8" s="11"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A9" s="27" t="s">
-        <v>95</v>
+      <c r="A9" s="24" t="s">
+        <v>97</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>36</v>
+        <v>172</v>
       </c>
       <c r="C9" s="25" t="s">
         <v>3</v>
       </c>
       <c r="D9" s="29" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E9" s="26" t="s">
-        <v>37</v>
+        <v>186</v>
       </c>
       <c r="F9" s="26" t="s">
-        <v>37</v>
+        <v>186</v>
       </c>
       <c r="G9" s="26" t="s">
-        <v>37</v>
+        <v>186</v>
       </c>
       <c r="H9" s="11"/>
       <c r="I9" s="11"/>
@@ -2333,22 +2342,22 @@
         <v>95</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C10" s="25" t="s">
         <v>3</v>
       </c>
       <c r="D10" s="29" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E10" s="26" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F10" s="26" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="G10" s="26" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="H10" s="11"/>
       <c r="I10" s="11"/>
@@ -2361,22 +2370,22 @@
         <v>95</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C11" s="25" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D11" s="29" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E11" s="26" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F11" s="26" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G11" s="26" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="H11" s="11"/>
       <c r="I11" s="11"/>
@@ -2389,22 +2398,22 @@
         <v>95</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C12" s="25" t="s">
         <v>5</v>
       </c>
       <c r="D12" s="29" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E12" s="26" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F12" s="26" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="G12" s="26" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="H12" s="11"/>
       <c r="I12" s="11"/>
@@ -2417,22 +2426,22 @@
         <v>95</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C13" s="25" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D13" s="29" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E13" s="26" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F13" s="26" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G13" s="26" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="H13" s="11"/>
       <c r="I13" s="11"/>
@@ -2445,22 +2454,22 @@
         <v>95</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C14" s="25" t="s">
         <v>4</v>
       </c>
       <c r="D14" s="29" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E14" s="26" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F14" s="26" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="G14" s="26" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="H14" s="11"/>
       <c r="I14" s="11"/>
@@ -2473,22 +2482,22 @@
         <v>95</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>173</v>
+        <v>46</v>
       </c>
       <c r="C15" s="25" t="s">
         <v>4</v>
       </c>
       <c r="D15" s="29" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E15" s="26" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F15" s="26" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G15" s="26" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H15" s="11"/>
       <c r="I15" s="11"/>
@@ -2501,22 +2510,22 @@
         <v>95</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C16" s="25" t="s">
         <v>4</v>
       </c>
       <c r="D16" s="29" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E16" s="26" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F16" s="26" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G16" s="26" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H16" s="11"/>
       <c r="I16" s="11"/>
@@ -2529,22 +2538,22 @@
         <v>95</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>50</v>
+        <v>174</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D17" s="29" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E17" s="26" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F17" s="26" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="G17" s="26" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="H17" s="11"/>
       <c r="I17" s="11"/>
@@ -2557,22 +2566,22 @@
         <v>95</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>175</v>
+        <v>50</v>
       </c>
       <c r="C18" s="25" t="s">
         <v>3</v>
       </c>
       <c r="D18" s="29" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E18" s="26" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F18" s="26" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G18" s="26" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H18" s="11"/>
       <c r="I18" s="11"/>
@@ -2585,22 +2594,22 @@
         <v>95</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>53</v>
+        <v>175</v>
       </c>
       <c r="C19" s="25" t="s">
         <v>3</v>
       </c>
       <c r="D19" s="29" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E19" s="26" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F19" s="26" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G19" s="26" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H19" s="11"/>
       <c r="I19" s="11"/>
@@ -2613,22 +2622,22 @@
         <v>95</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>176</v>
+        <v>53</v>
       </c>
       <c r="C20" s="25" t="s">
         <v>3</v>
       </c>
       <c r="D20" s="29" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E20" s="26" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F20" s="26" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G20" s="26" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H20" s="11"/>
       <c r="I20" s="11"/>
@@ -2637,26 +2646,26 @@
       <c r="L20" s="11"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A21" s="24" t="s">
-        <v>94</v>
+      <c r="A21" s="27" t="s">
+        <v>95</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C21" s="25" t="s">
         <v>3</v>
       </c>
       <c r="D21" s="29" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E21" s="26" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F21" s="26" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G21" s="26" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H21" s="11"/>
       <c r="I21" s="11"/>
@@ -2669,22 +2678,22 @@
         <v>94</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C22" s="25" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D22" s="29" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E22" s="26" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F22" s="26" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G22" s="26" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H22" s="11"/>
       <c r="I22" s="11"/>
@@ -2697,22 +2706,24 @@
         <v>94</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="C23" s="25"/>
+        <v>178</v>
+      </c>
+      <c r="C23" s="25" t="s">
+        <v>5</v>
+      </c>
       <c r="D23" s="29" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E23" s="26" t="s">
-        <v>272</v>
+        <v>57</v>
       </c>
       <c r="F23" s="26" t="s">
-        <v>272</v>
+        <v>57</v>
       </c>
       <c r="G23" s="26" t="s">
-        <v>272</v>
-      </c>
-      <c r="H23" s="26"/>
+        <v>57</v>
+      </c>
+      <c r="H23" s="11"/>
       <c r="I23" s="11"/>
       <c r="J23" s="11"/>
       <c r="K23" s="11"/>
@@ -2723,22 +2734,22 @@
         <v>94</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>179</v>
+        <v>15</v>
       </c>
       <c r="C24" s="25"/>
       <c r="D24" s="29" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E24" s="26" t="s">
-        <v>35</v>
+        <v>272</v>
       </c>
       <c r="F24" s="26" t="s">
-        <v>35</v>
+        <v>272</v>
       </c>
       <c r="G24" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="H24" s="11"/>
+        <v>272</v>
+      </c>
+      <c r="H24" s="26"/>
       <c r="I24" s="11"/>
       <c r="J24" s="11"/>
       <c r="K24" s="11"/>
@@ -2749,22 +2760,20 @@
         <v>94</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="C25" s="25" t="s">
-        <v>4</v>
-      </c>
+        <v>179</v>
+      </c>
+      <c r="C25" s="25"/>
       <c r="D25" s="29" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E25" s="26" t="s">
-        <v>58</v>
+        <v>35</v>
       </c>
       <c r="F25" s="26" t="s">
-        <v>58</v>
+        <v>35</v>
       </c>
       <c r="G25" s="26" t="s">
-        <v>58</v>
+        <v>35</v>
       </c>
       <c r="H25" s="11"/>
       <c r="I25" s="11"/>
@@ -2773,26 +2782,26 @@
       <c r="L25" s="11"/>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A26" s="27" t="s">
-        <v>17</v>
+      <c r="A26" s="24" t="s">
+        <v>94</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C26" s="25" t="s">
-        <v>63</v>
+        <v>4</v>
       </c>
       <c r="D26" s="29" t="s">
-        <v>211</v>
-      </c>
-      <c r="E26" s="28" t="s">
-        <v>234</v>
-      </c>
-      <c r="F26" s="28" t="s">
-        <v>234</v>
-      </c>
-      <c r="G26" s="28" t="s">
-        <v>234</v>
+        <v>210</v>
+      </c>
+      <c r="E26" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="F26" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="G26" s="26" t="s">
+        <v>58</v>
       </c>
       <c r="H26" s="11"/>
       <c r="I26" s="11"/>
@@ -2801,26 +2810,26 @@
       <c r="L26" s="11"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A27" s="24" t="s">
-        <v>93</v>
+      <c r="A27" s="27" t="s">
+        <v>17</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>180</v>
+        <v>18</v>
       </c>
       <c r="C27" s="25" t="s">
         <v>63</v>
       </c>
       <c r="D27" s="29" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="E27" s="28" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F27" s="28" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="G27" s="28" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="H27" s="11"/>
       <c r="I27" s="11"/>
@@ -2833,22 +2842,22 @@
         <v>93</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C28" s="25" t="s">
-        <v>4</v>
+        <v>63</v>
       </c>
       <c r="D28" s="29" t="s">
-        <v>220</v>
-      </c>
-      <c r="E28" s="26" t="s">
-        <v>233</v>
-      </c>
-      <c r="F28" s="26" t="s">
-        <v>233</v>
-      </c>
-      <c r="G28" s="26" t="s">
-        <v>233</v>
+        <v>219</v>
+      </c>
+      <c r="E28" s="28" t="s">
+        <v>235</v>
+      </c>
+      <c r="F28" s="28" t="s">
+        <v>235</v>
+      </c>
+      <c r="G28" s="28" t="s">
+        <v>235</v>
       </c>
       <c r="H28" s="11"/>
       <c r="I28" s="11"/>
@@ -2857,26 +2866,26 @@
       <c r="L28" s="11"/>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A29" s="27" t="s">
-        <v>92</v>
+      <c r="A29" s="24" t="s">
+        <v>93</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>20</v>
+        <v>181</v>
       </c>
       <c r="C29" s="25" t="s">
-        <v>59</v>
+        <v>4</v>
       </c>
       <c r="D29" s="29" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="E29" s="26" t="s">
-        <v>60</v>
+        <v>233</v>
       </c>
       <c r="F29" s="26" t="s">
-        <v>60</v>
+        <v>233</v>
       </c>
       <c r="G29" s="26" t="s">
-        <v>60</v>
+        <v>233</v>
       </c>
       <c r="H29" s="11"/>
       <c r="I29" s="11"/>
@@ -2889,22 +2898,22 @@
         <v>92</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C30" s="25" t="s">
-        <v>98</v>
+        <v>59</v>
       </c>
       <c r="D30" s="29" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="E30" s="26" t="s">
-        <v>275</v>
+        <v>60</v>
       </c>
       <c r="F30" s="26" t="s">
-        <v>275</v>
+        <v>60</v>
       </c>
       <c r="G30" s="26" t="s">
-        <v>275</v>
+        <v>60</v>
       </c>
       <c r="H30" s="11"/>
       <c r="I30" s="11"/>
@@ -2917,22 +2926,22 @@
         <v>92</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C31" s="25" t="s">
-        <v>187</v>
+        <v>98</v>
       </c>
       <c r="D31" s="29" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E31" s="26" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="F31" s="26" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="G31" s="26" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="H31" s="11"/>
       <c r="I31" s="11"/>
@@ -2945,22 +2954,22 @@
         <v>92</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="C32" s="25" t="s">
-        <v>63</v>
+        <v>187</v>
       </c>
       <c r="D32" s="29" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E32" s="26" t="s">
-        <v>236</v>
+        <v>278</v>
       </c>
       <c r="F32" s="26" t="s">
-        <v>236</v>
+        <v>278</v>
       </c>
       <c r="G32" s="26" t="s">
-        <v>236</v>
+        <v>278</v>
       </c>
       <c r="H32" s="11"/>
       <c r="I32" s="11"/>
@@ -2973,22 +2982,22 @@
         <v>92</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C33" s="25" t="s">
         <v>63</v>
       </c>
       <c r="D33" s="29" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E33" s="26" t="s">
-        <v>64</v>
+        <v>236</v>
       </c>
       <c r="F33" s="26" t="s">
-        <v>64</v>
+        <v>236</v>
       </c>
       <c r="G33" s="26" t="s">
-        <v>64</v>
+        <v>236</v>
       </c>
       <c r="H33" s="11"/>
       <c r="I33" s="11"/>
@@ -3001,22 +3010,22 @@
         <v>92</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C34" s="25" t="s">
         <v>63</v>
       </c>
       <c r="D34" s="29" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E34" s="26" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F34" s="26" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G34" s="26" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H34" s="11"/>
       <c r="I34" s="11"/>
@@ -3029,52 +3038,52 @@
         <v>92</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C35" s="25" t="s">
         <v>63</v>
       </c>
       <c r="D35" s="29" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E35" s="26" t="s">
-        <v>273</v>
+        <v>66</v>
       </c>
       <c r="F35" s="26" t="s">
-        <v>273</v>
+        <v>66</v>
       </c>
       <c r="G35" s="26" t="s">
-        <v>273</v>
-      </c>
-      <c r="H35" s="26"/>
+        <v>66</v>
+      </c>
+      <c r="H35" s="11"/>
       <c r="I35" s="11"/>
       <c r="J35" s="11"/>
       <c r="K35" s="11"/>
       <c r="L35" s="11"/>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A36" s="24" t="s">
-        <v>90</v>
+      <c r="A36" s="27" t="s">
+        <v>92</v>
       </c>
       <c r="B36" s="11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C36" s="25" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="D36" s="29" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="E36" s="26" t="s">
-        <v>70</v>
+        <v>273</v>
       </c>
       <c r="F36" s="26" t="s">
-        <v>70</v>
+        <v>273</v>
       </c>
       <c r="G36" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="H36" s="11"/>
+        <v>273</v>
+      </c>
+      <c r="H36" s="26"/>
       <c r="I36" s="11"/>
       <c r="J36" s="11"/>
       <c r="K36" s="11"/>
@@ -3085,22 +3094,22 @@
         <v>90</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>182</v>
+        <v>68</v>
       </c>
       <c r="C37" s="25" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D37" s="29" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E37" s="26" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F37" s="26" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G37" s="26" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="H37" s="11"/>
       <c r="I37" s="11"/>
@@ -3113,22 +3122,22 @@
         <v>90</v>
       </c>
       <c r="B38" s="11" t="s">
-        <v>73</v>
+        <v>182</v>
       </c>
       <c r="C38" s="25" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="D38" s="29" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E38" s="26" t="s">
-        <v>237</v>
-      </c>
-      <c r="F38" s="11" t="s">
-        <v>241</v>
-      </c>
-      <c r="G38" s="11" t="s">
-        <v>241</v>
+        <v>72</v>
+      </c>
+      <c r="F38" s="26" t="s">
+        <v>72</v>
+      </c>
+      <c r="G38" s="26" t="s">
+        <v>72</v>
       </c>
       <c r="H38" s="11"/>
       <c r="I38" s="11"/>
@@ -3141,22 +3150,22 @@
         <v>90</v>
       </c>
       <c r="B39" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C39" s="25" t="s">
         <v>4</v>
       </c>
       <c r="D39" s="29" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E39" s="26" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="H39" s="11"/>
       <c r="I39" s="11"/>
@@ -3169,22 +3178,22 @@
         <v>90</v>
       </c>
       <c r="B40" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C40" s="25" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D40" s="29" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E40" s="26" t="s">
-        <v>76</v>
-      </c>
-      <c r="F40" s="26" t="s">
-        <v>76</v>
-      </c>
-      <c r="G40" s="26" t="s">
-        <v>76</v>
+        <v>238</v>
+      </c>
+      <c r="F40" s="11" t="s">
+        <v>242</v>
+      </c>
+      <c r="G40" s="11" t="s">
+        <v>242</v>
       </c>
       <c r="H40" s="11"/>
       <c r="I40" s="11"/>
@@ -3197,22 +3206,22 @@
         <v>90</v>
       </c>
       <c r="B41" s="11" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C41" s="25" t="s">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="D41" s="29" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E41" s="26" t="s">
-        <v>78</v>
-      </c>
-      <c r="F41" s="11" t="s">
-        <v>243</v>
-      </c>
-      <c r="G41" s="11" t="s">
-        <v>243</v>
+        <v>76</v>
+      </c>
+      <c r="F41" s="26" t="s">
+        <v>76</v>
+      </c>
+      <c r="G41" s="26" t="s">
+        <v>76</v>
       </c>
       <c r="H41" s="11"/>
       <c r="I41" s="11"/>
@@ -3221,26 +3230,26 @@
       <c r="L41" s="11"/>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A42" s="27" t="s">
-        <v>91</v>
+      <c r="A42" s="24" t="s">
+        <v>90</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C42" s="25" t="s">
-        <v>69</v>
+        <v>33</v>
       </c>
       <c r="D42" s="29" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E42" s="26" t="s">
-        <v>80</v>
-      </c>
-      <c r="F42" s="26" t="s">
-        <v>80</v>
-      </c>
-      <c r="G42" s="26" t="s">
-        <v>80</v>
+        <v>78</v>
+      </c>
+      <c r="F42" s="11" t="s">
+        <v>243</v>
+      </c>
+      <c r="G42" s="11" t="s">
+        <v>243</v>
       </c>
       <c r="H42" s="11"/>
       <c r="I42" s="11"/>
@@ -3253,22 +3262,22 @@
         <v>91</v>
       </c>
       <c r="B43" s="11" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C43" s="25" t="s">
         <v>69</v>
       </c>
       <c r="D43" s="29" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E43" s="26" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F43" s="26" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G43" s="26" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="H43" s="11"/>
       <c r="I43" s="11"/>
@@ -3281,22 +3290,22 @@
         <v>91</v>
       </c>
       <c r="B44" s="11" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C44" s="25" t="s">
-        <v>4</v>
+        <v>69</v>
       </c>
       <c r="D44" s="29" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E44" s="26" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F44" s="26" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="G44" s="26" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="H44" s="11"/>
       <c r="I44" s="11"/>
@@ -3309,22 +3318,22 @@
         <v>91</v>
       </c>
       <c r="B45" s="11" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C45" s="25" t="s">
         <v>4</v>
       </c>
       <c r="D45" s="29" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E45" s="26" t="s">
-        <v>274</v>
+        <v>84</v>
       </c>
       <c r="F45" s="26" t="s">
-        <v>274</v>
+        <v>84</v>
       </c>
       <c r="G45" s="26" t="s">
-        <v>274</v>
+        <v>84</v>
       </c>
       <c r="H45" s="11"/>
       <c r="I45" s="11"/>
@@ -3333,26 +3342,26 @@
       <c r="L45" s="11"/>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A46" s="24" t="s">
-        <v>111</v>
+      <c r="A46" s="27" t="s">
+        <v>91</v>
       </c>
       <c r="B46" s="11" t="s">
-        <v>183</v>
+        <v>85</v>
       </c>
       <c r="C46" s="25" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D46" s="29" t="s">
-        <v>231</v>
-      </c>
-      <c r="E46" s="28" t="s">
-        <v>239</v>
-      </c>
-      <c r="F46" s="28" t="s">
-        <v>239</v>
-      </c>
-      <c r="G46" s="28" t="s">
-        <v>239</v>
+        <v>230</v>
+      </c>
+      <c r="E46" s="26" t="s">
+        <v>274</v>
+      </c>
+      <c r="F46" s="26" t="s">
+        <v>274</v>
+      </c>
+      <c r="G46" s="26" t="s">
+        <v>274</v>
       </c>
       <c r="H46" s="11"/>
       <c r="I46" s="11"/>
@@ -3365,22 +3374,22 @@
         <v>111</v>
       </c>
       <c r="B47" s="11" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C47" s="25" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D47" s="29" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E47" s="28" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F47" s="28" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G47" s="28" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="H47" s="11"/>
       <c r="I47" s="11"/>
@@ -3389,13 +3398,27 @@
       <c r="L47" s="11"/>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A48" s="11"/>
-      <c r="B48" s="28"/>
-      <c r="C48" s="25"/>
-      <c r="D48" s="26"/>
-      <c r="E48" s="28"/>
-      <c r="F48" s="11"/>
-      <c r="G48" s="11"/>
+      <c r="A48" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="B48" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="C48" s="25" t="s">
+        <v>71</v>
+      </c>
+      <c r="D48" s="29" t="s">
+        <v>232</v>
+      </c>
+      <c r="E48" s="28" t="s">
+        <v>240</v>
+      </c>
+      <c r="F48" s="28" t="s">
+        <v>240</v>
+      </c>
+      <c r="G48" s="28" t="s">
+        <v>240</v>
+      </c>
       <c r="H48" s="11"/>
       <c r="I48" s="11"/>
       <c r="J48" s="11"/>
@@ -4130,18 +4153,32 @@
       <c r="K100" s="11"/>
       <c r="L100" s="11"/>
     </row>
+    <row r="101" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A101" s="11"/>
+      <c r="B101" s="28"/>
+      <c r="C101" s="25"/>
+      <c r="D101" s="26"/>
+      <c r="E101" s="28"/>
+      <c r="F101" s="11"/>
+      <c r="G101" s="11"/>
+      <c r="H101" s="11"/>
+      <c r="I101" s="11"/>
+      <c r="J101" s="11"/>
+      <c r="K101" s="11"/>
+      <c r="L101" s="11"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
-  <conditionalFormatting sqref="B2:B6">
+  <conditionalFormatting sqref="B2:B7">
     <cfRule type="duplicateValues" dxfId="3" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2:B47">
+  <conditionalFormatting sqref="B2:B48">
     <cfRule type="duplicateValues" dxfId="2" priority="5"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B7:B47">
+  <conditionalFormatting sqref="B8:B48">
     <cfRule type="duplicateValues" dxfId="1" priority="6"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D47">
+  <conditionalFormatting sqref="D2:D48">
     <cfRule type="duplicateValues" dxfId="0" priority="7"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Apply workbook sign conventions to RCA energy analysis
</commit_message>
<xml_diff>
--- a/eBus_Functions/Post_Processing/Root_Cause_Analysis_Work/info/eBus_Model_Info.xlsx
+++ b/eBus_Functions/Post_Processing/Root_Cause_Analysis_Work/info/eBus_Model_Info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TempData\Github\eBus_Tool\eBus_Functions\Post_Processing\Root_Cause_Analysis_Work\info\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDB3083A-0D9A-4053-A0E4-13B87157D318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7272B2ED-3F53-48A5-9A27-83D7642A9B46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Block_Diagram" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="307">
   <si>
     <t>Driver</t>
   </si>
@@ -909,6 +909,45 @@
   </si>
   <si>
     <t>logout.sec</t>
+  </si>
+  <si>
+    <t>Battery Current (Positive for Charge and Negative for Discharge)</t>
+  </si>
+  <si>
+    <t>Battery Power (Positive for Charge and Negative for Discharge)</t>
+  </si>
+  <si>
+    <t>Electric Motor 1 Demand Torque (Positive for Driving Torque and Negative for Recuperation Torque)</t>
+  </si>
+  <si>
+    <t>Electric Motor 2 Demand Torque (Positive for Driving Torque and Negative for Recuperation Torque)</t>
+  </si>
+  <si>
+    <t>Motor 1 Actual Torque (Positive for Driving Torque and Negative for Recuperation Torque)</t>
+  </si>
+  <si>
+    <t>Motor 2 Actual Torque (Positive for Driving Torque and Negative for Recuperation Torque)</t>
+  </si>
+  <si>
+    <t>Motor 1 Electrical Power (Positive for Driving Power and Negative for Recuperation Power)</t>
+  </si>
+  <si>
+    <t>Motor 2 Electrical Power (Positive for Driving Power and Negative for Recuperation Power)</t>
+  </si>
+  <si>
+    <t>Motor 1 Max Available Torque (Positive for Driving Torque and Negative for Recuperation Torque)</t>
+  </si>
+  <si>
+    <t>Motor 1 Min Available Torque (Positive for Driving Torque and Negative for Recuperation Torque)</t>
+  </si>
+  <si>
+    <t>Motor 2 Max Available Torque (Positive for Driving Torque and Negative for Recuperation Torque)</t>
+  </si>
+  <si>
+    <t>Motor 2 Min Available Torque (Positive for Driving Torque and Negative for Recuperation Torque)</t>
+  </si>
+  <si>
+    <t>Gear Box Output Torque (Positive for Driving Torque and Negative for Recuperation Torque)</t>
   </si>
 </sst>
 </file>
@@ -1222,9 +1261,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1238,6 +1274,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1642,7 +1681,7 @@
     </row>
     <row r="29" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G29" s="6"/>
-      <c r="H29" s="31" t="s">
+      <c r="H29" s="36" t="s">
         <v>6</v>
       </c>
       <c r="I29" s="7" t="s">
@@ -1651,14 +1690,14 @@
     </row>
     <row r="30" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G30" s="8"/>
-      <c r="H30" s="32"/>
+      <c r="H30" s="31"/>
       <c r="I30" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="31" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G31" s="9"/>
-      <c r="H31" s="33"/>
+      <c r="H31" s="32"/>
       <c r="I31" s="2" t="s">
         <v>32</v>
       </c>
@@ -1667,7 +1706,7 @@
       <c r="G32" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="H32" s="34" t="s">
+      <c r="H32" s="33" t="s">
         <v>0</v>
       </c>
       <c r="I32" s="7" t="s">
@@ -1678,7 +1717,7 @@
       <c r="G33" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="H33" s="35"/>
+      <c r="H33" s="34"/>
       <c r="I33" s="1" t="s">
         <v>12</v>
       </c>
@@ -1687,35 +1726,35 @@
       <c r="G34" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="H34" s="35"/>
+      <c r="H34" s="34"/>
       <c r="I34" s="1"/>
     </row>
     <row r="35" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G35" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="H35" s="35"/>
+      <c r="H35" s="34"/>
       <c r="I35" s="1"/>
     </row>
     <row r="36" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G36" s="8" t="s">
         <v>179</v>
       </c>
-      <c r="H36" s="35"/>
+      <c r="H36" s="34"/>
       <c r="I36" s="1"/>
     </row>
     <row r="37" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G37" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="H37" s="36"/>
+      <c r="H37" s="35"/>
       <c r="I37" s="2"/>
     </row>
     <row r="38" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G38" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="H38" s="31" t="s">
+      <c r="H38" s="36" t="s">
         <v>2</v>
       </c>
       <c r="I38" s="7" t="s">
@@ -1726,7 +1765,7 @@
       <c r="G39" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="H39" s="33"/>
+      <c r="H39" s="32"/>
       <c r="I39" s="2" t="s">
         <v>172</v>
       </c>
@@ -1735,7 +1774,7 @@
       <c r="G40" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="H40" s="34" t="s">
+      <c r="H40" s="33" t="s">
         <v>106</v>
       </c>
       <c r="I40" s="7" t="s">
@@ -1746,77 +1785,77 @@
       <c r="G41" s="8" t="s">
         <v>172</v>
       </c>
-      <c r="H41" s="35"/>
+      <c r="H41" s="34"/>
       <c r="I41" s="1" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="42" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G42" s="8"/>
-      <c r="H42" s="35"/>
+      <c r="H42" s="34"/>
       <c r="I42" s="1" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="43" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G43" s="8"/>
-      <c r="H43" s="35"/>
+      <c r="H43" s="34"/>
       <c r="I43" s="1" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="44" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G44" s="8"/>
-      <c r="H44" s="35"/>
+      <c r="H44" s="34"/>
       <c r="I44" s="1" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="45" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G45" s="8"/>
-      <c r="H45" s="35"/>
+      <c r="H45" s="34"/>
       <c r="I45" s="1" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="46" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G46" s="8"/>
-      <c r="H46" s="35"/>
+      <c r="H46" s="34"/>
       <c r="I46" s="1" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="47" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G47" s="8"/>
-      <c r="H47" s="35"/>
+      <c r="H47" s="34"/>
       <c r="I47" s="1" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="48" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G48" s="8"/>
-      <c r="H48" s="35"/>
+      <c r="H48" s="34"/>
       <c r="I48" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="49" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G49" s="8"/>
-      <c r="H49" s="35"/>
+      <c r="H49" s="34"/>
       <c r="I49" s="1" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="50" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G50" s="8"/>
-      <c r="H50" s="35"/>
+      <c r="H50" s="34"/>
       <c r="I50" s="1" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="51" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G51" s="9"/>
-      <c r="H51" s="36"/>
+      <c r="H51" s="35"/>
       <c r="I51" s="2" t="s">
         <v>176</v>
       </c>
@@ -1825,7 +1864,7 @@
       <c r="G52" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="H52" s="31" t="s">
+      <c r="H52" s="36" t="s">
         <v>107</v>
       </c>
       <c r="I52" s="7" t="s">
@@ -1836,28 +1875,28 @@
       <c r="G53" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="H53" s="32"/>
+      <c r="H53" s="31"/>
       <c r="I53" s="1" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="54" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G54" s="8"/>
-      <c r="H54" s="32"/>
+      <c r="H54" s="31"/>
       <c r="I54" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="55" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G55" s="8"/>
-      <c r="H55" s="32"/>
+      <c r="H55" s="31"/>
       <c r="I55" s="1" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="56" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G56" s="8"/>
-      <c r="H56" s="32"/>
+      <c r="H56" s="31"/>
       <c r="I56" s="1" t="s">
         <v>16</v>
       </c>
@@ -1877,7 +1916,7 @@
       <c r="G58" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="H58" s="34" t="s">
+      <c r="H58" s="33" t="s">
         <v>108</v>
       </c>
       <c r="I58" s="7" t="s">
@@ -1886,7 +1925,7 @@
     </row>
     <row r="59" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G59" s="8"/>
-      <c r="H59" s="35"/>
+      <c r="H59" s="34"/>
       <c r="I59" s="1" t="s">
         <v>181</v>
       </c>
@@ -1895,7 +1934,7 @@
       <c r="G60" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="H60" s="31" t="s">
+      <c r="H60" s="36" t="s">
         <v>19</v>
       </c>
       <c r="I60" s="7" t="s">
@@ -1906,42 +1945,42 @@
       <c r="G61" s="8" t="s">
         <v>180</v>
       </c>
-      <c r="H61" s="32"/>
+      <c r="H61" s="31"/>
       <c r="I61" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="62" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G62" s="8"/>
-      <c r="H62" s="32"/>
+      <c r="H62" s="31"/>
       <c r="I62" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="63" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G63" s="8"/>
-      <c r="H63" s="32"/>
+      <c r="H63" s="31"/>
       <c r="I63" s="1" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="64" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G64" s="8"/>
-      <c r="H64" s="32"/>
+      <c r="H64" s="31"/>
       <c r="I64" s="1" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="65" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G65" s="8"/>
-      <c r="H65" s="32"/>
+      <c r="H65" s="31"/>
       <c r="I65" s="1" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="66" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G66" s="9"/>
-      <c r="H66" s="33"/>
+      <c r="H66" s="32"/>
       <c r="I66" s="2" t="s">
         <v>67</v>
       </c>
@@ -1950,7 +1989,7 @@
       <c r="G67" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="H67" s="32" t="s">
+      <c r="H67" s="31" t="s">
         <v>109</v>
       </c>
       <c r="I67" s="1" t="s">
@@ -1959,35 +1998,35 @@
     </row>
     <row r="68" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G68" s="8"/>
-      <c r="H68" s="32"/>
+      <c r="H68" s="31"/>
       <c r="I68" s="1" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="69" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G69" s="8"/>
-      <c r="H69" s="32"/>
+      <c r="H69" s="31"/>
       <c r="I69" s="1" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="70" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G70" s="8"/>
-      <c r="H70" s="32"/>
+      <c r="H70" s="31"/>
       <c r="I70" s="1" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="71" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G71" s="8"/>
-      <c r="H71" s="32"/>
+      <c r="H71" s="31"/>
       <c r="I71" s="1" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="72" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G72" s="9"/>
-      <c r="H72" s="33"/>
+      <c r="H72" s="32"/>
       <c r="I72" s="2" t="s">
         <v>77</v>
       </c>
@@ -1996,7 +2035,7 @@
       <c r="G73" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="H73" s="34" t="s">
+      <c r="H73" s="33" t="s">
         <v>110</v>
       </c>
       <c r="I73" s="7" t="s">
@@ -2007,28 +2046,28 @@
       <c r="G74" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="H74" s="35"/>
+      <c r="H74" s="34"/>
       <c r="I74" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="75" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G75" s="8"/>
-      <c r="H75" s="35"/>
+      <c r="H75" s="34"/>
       <c r="I75" s="1" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="76" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G76" s="9"/>
-      <c r="H76" s="36"/>
+      <c r="H76" s="35"/>
       <c r="I76" s="2" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="77" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G77" s="8"/>
-      <c r="H77" s="32" t="s">
+      <c r="H77" s="31" t="s">
         <v>111</v>
       </c>
       <c r="I77" s="1" t="s">
@@ -2037,30 +2076,30 @@
     </row>
     <row r="78" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G78" s="8"/>
-      <c r="H78" s="32"/>
+      <c r="H78" s="31"/>
       <c r="I78" s="1" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="79" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G79" s="9"/>
-      <c r="H79" s="33"/>
+      <c r="H79" s="32"/>
       <c r="I79" s="2" t="s">
         <v>185</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="H29:H31"/>
+    <mergeCell ref="H32:H37"/>
+    <mergeCell ref="H38:H39"/>
+    <mergeCell ref="H40:H51"/>
+    <mergeCell ref="H58:H59"/>
     <mergeCell ref="H67:H72"/>
     <mergeCell ref="H73:H76"/>
     <mergeCell ref="H52:H56"/>
     <mergeCell ref="H60:H66"/>
     <mergeCell ref="H77:H79"/>
-    <mergeCell ref="H29:H31"/>
-    <mergeCell ref="H32:H37"/>
-    <mergeCell ref="H38:H39"/>
-    <mergeCell ref="H40:H51"/>
-    <mergeCell ref="H58:H59"/>
   </mergeCells>
   <conditionalFormatting sqref="I29:I79 G29:G79">
     <cfRule type="duplicateValues" dxfId="4" priority="1"/>
@@ -2077,7 +2116,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28" style="20" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.88671875" style="20" customWidth="1"/>
     <col min="3" max="3" width="19" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24.6640625" style="21" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="46.44140625" style="20" bestFit="1" customWidth="1"/>
@@ -2286,7 +2325,7 @@
         <v>97</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>171</v>
+        <v>296</v>
       </c>
       <c r="C8" s="25" t="s">
         <v>3</v>
@@ -2314,7 +2353,7 @@
         <v>97</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>172</v>
+        <v>297</v>
       </c>
       <c r="C9" s="25" t="s">
         <v>3</v>
@@ -2342,7 +2381,7 @@
         <v>95</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>36</v>
+        <v>298</v>
       </c>
       <c r="C10" s="25" t="s">
         <v>3</v>
@@ -2370,7 +2409,7 @@
         <v>95</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>38</v>
+        <v>299</v>
       </c>
       <c r="C11" s="25" t="s">
         <v>3</v>
@@ -2454,7 +2493,7 @@
         <v>95</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>44</v>
+        <v>300</v>
       </c>
       <c r="C14" s="25" t="s">
         <v>4</v>
@@ -2482,7 +2521,7 @@
         <v>95</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>46</v>
+        <v>301</v>
       </c>
       <c r="C15" s="25" t="s">
         <v>4</v>
@@ -2566,7 +2605,7 @@
         <v>95</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>50</v>
+        <v>302</v>
       </c>
       <c r="C18" s="25" t="s">
         <v>3</v>
@@ -2594,7 +2633,7 @@
         <v>95</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>175</v>
+        <v>303</v>
       </c>
       <c r="C19" s="25" t="s">
         <v>3</v>
@@ -2622,7 +2661,7 @@
         <v>95</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>53</v>
+        <v>304</v>
       </c>
       <c r="C20" s="25" t="s">
         <v>3</v>
@@ -2650,7 +2689,7 @@
         <v>95</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>176</v>
+        <v>305</v>
       </c>
       <c r="C21" s="25" t="s">
         <v>3</v>
@@ -2678,7 +2717,7 @@
         <v>94</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>177</v>
+        <v>306</v>
       </c>
       <c r="C22" s="25" t="s">
         <v>3</v>
@@ -3094,7 +3133,7 @@
         <v>90</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>68</v>
+        <v>294</v>
       </c>
       <c r="C37" s="25" t="s">
         <v>69</v>
@@ -3150,7 +3189,7 @@
         <v>90</v>
       </c>
       <c r="B39" s="11" t="s">
-        <v>73</v>
+        <v>295</v>
       </c>
       <c r="C39" s="25" t="s">
         <v>4</v>

</xml_diff>

<commit_message>
Use workbook specifications in subsystem RCA
</commit_message>
<xml_diff>
--- a/eBus_Functions/Post_Processing/Root_Cause_Analysis_Work/info/eBus_Model_Info.xlsx
+++ b/eBus_Functions/Post_Processing/Root_Cause_Analysis_Work/info/eBus_Model_Info.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TempData\Github\eBus_Tool\eBus_Functions\Post_Processing\Root_Cause_Analysis_Work\info\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30AB63F5-F1F8-493A-A929-D72CCA2CA18E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8325D24C-37B5-484E-BEFB-0DD5230CE88D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Block_Diagram" sheetId="1" r:id="rId1"/>
     <sheet name="Signal_Evaluation" sheetId="2" r:id="rId2"/>
     <sheet name="Specifications" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="683" uniqueCount="323">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="324">
   <si>
     <t>Driver</t>
   </si>
@@ -374,9 +375,6 @@
     <t>rpm</t>
   </si>
   <si>
-    <t>Wheel Rolling Resistance</t>
-  </si>
-  <si>
     <t>Wheel Radius</t>
   </si>
   <si>
@@ -996,6 +994,12 @@
   </si>
   <si>
     <t>logout.MinAvlEmotTrq_Cval_CPC/2</t>
+  </si>
+  <si>
+    <t>Wheel Rolling Resistance Coefficient</t>
+  </si>
+  <si>
+    <t>m</t>
   </si>
 </sst>
 </file>
@@ -1159,7 +1163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1212,17 +1216,16 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1626,469 +1629,421 @@
       </c>
     </row>
     <row r="29" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G29" s="23"/>
       <c r="H29" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="I29" s="23" t="s">
+      <c r="I29" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="30" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G30" s="23"/>
       <c r="H30" s="24"/>
-      <c r="I30" s="23" t="s">
+      <c r="I30" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="31" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G31" s="23"/>
       <c r="H31" s="24"/>
-      <c r="I31" s="23" t="s">
+      <c r="I31" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="32" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G32" s="23" t="s">
+      <c r="G32" t="s">
         <v>21</v>
       </c>
       <c r="H32" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="I32" s="23" t="s">
+      <c r="I32" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="33" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G33" s="23" t="s">
+      <c r="G33" t="s">
         <v>29</v>
       </c>
       <c r="H33" s="25"/>
-      <c r="I33" s="23" t="s">
+      <c r="I33" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="34" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G34" s="23" t="s">
+      <c r="G34" t="s">
         <v>7</v>
       </c>
       <c r="H34" s="25"/>
-      <c r="I34" s="23"/>
     </row>
     <row r="35" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G35" s="23" t="s">
+      <c r="G35" t="s">
         <v>13</v>
       </c>
       <c r="H35" s="25"/>
-      <c r="I35" s="23"/>
     </row>
     <row r="36" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G36" s="23" t="s">
-        <v>179</v>
+      <c r="G36" t="s">
+        <v>178</v>
       </c>
       <c r="H36" s="25"/>
-      <c r="I36" s="23"/>
     </row>
     <row r="37" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G37" s="23" t="s">
+      <c r="G37" t="s">
         <v>14</v>
       </c>
       <c r="H37" s="25"/>
-      <c r="I37" s="23"/>
     </row>
     <row r="38" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G38" s="23" t="s">
+      <c r="G38" t="s">
         <v>11</v>
       </c>
       <c r="H38" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="I38" s="23" t="s">
+      <c r="I38" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="39" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="G39" t="s">
+        <v>12</v>
+      </c>
+      <c r="H39" s="24"/>
+      <c r="I39" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="39" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G39" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="H39" s="24"/>
-      <c r="I39" s="23" t="s">
-        <v>172</v>
-      </c>
-    </row>
     <row r="40" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G40" s="23"/>
       <c r="H40" s="24"/>
-      <c r="I40" s="23" t="s">
+      <c r="I40" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="41" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="H41" s="24"/>
+      <c r="I41" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="41" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G41" s="23"/>
-      <c r="H41" s="24"/>
-      <c r="I41" s="23" t="s">
-        <v>308</v>
-      </c>
-    </row>
     <row r="42" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G42" s="23"/>
       <c r="H42" s="24"/>
-      <c r="I42" s="23" t="s">
+      <c r="I42" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="43" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="H43" s="24"/>
+      <c r="I43" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="43" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G43" s="23"/>
-      <c r="H43" s="24"/>
-      <c r="I43" s="23" t="s">
-        <v>312</v>
-      </c>
-    </row>
     <row r="44" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G44" s="23"/>
       <c r="H44" s="24"/>
-      <c r="I44" s="23"/>
     </row>
     <row r="45" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G45" s="23"/>
       <c r="H45" s="24"/>
-      <c r="I45" s="23"/>
     </row>
     <row r="46" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G46" s="23"/>
       <c r="H46" s="24"/>
-      <c r="I46" s="23"/>
     </row>
     <row r="47" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G47" s="23"/>
       <c r="H47" s="24"/>
-      <c r="I47" s="23"/>
     </row>
     <row r="48" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G48" s="23"/>
       <c r="H48" s="22"/>
-      <c r="I48" s="23"/>
     </row>
     <row r="49" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G49" s="23" t="s">
-        <v>171</v>
+      <c r="G49" t="s">
+        <v>170</v>
       </c>
       <c r="H49" s="25" t="s">
         <v>106</v>
       </c>
-      <c r="I49" s="23" t="s">
+      <c r="I49" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="50" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G50" s="23" t="s">
+      <c r="G50" t="s">
+        <v>171</v>
+      </c>
+      <c r="H50" s="25"/>
+      <c r="I50" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="51" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="G51" t="s">
+        <v>308</v>
+      </c>
+      <c r="H51" s="25"/>
+      <c r="I51" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="52" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="G52" t="s">
+        <v>309</v>
+      </c>
+      <c r="H52" s="25"/>
+      <c r="I52" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="53" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="H53" s="25"/>
+      <c r="I53" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="54" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="H54" s="25"/>
+      <c r="I54" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="55" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="H55" s="25"/>
+      <c r="I55" t="s">
         <v>172</v>
       </c>
-      <c r="H50" s="25"/>
-      <c r="I50" s="23" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="51" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G51" s="23" t="s">
-        <v>309</v>
-      </c>
-      <c r="H51" s="25"/>
-      <c r="I51" s="23" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="52" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G52" s="23" t="s">
-        <v>310</v>
-      </c>
-      <c r="H52" s="25"/>
-      <c r="I52" s="23" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="53" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G53" s="23"/>
-      <c r="H53" s="25"/>
-      <c r="I53" s="23" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="54" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G54" s="23"/>
-      <c r="H54" s="25"/>
-      <c r="I54" s="23" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="55" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G55" s="23"/>
-      <c r="H55" s="25"/>
-      <c r="I55" s="23" t="s">
+    </row>
+    <row r="56" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="H56" s="25"/>
+      <c r="I56" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="56" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G56" s="23"/>
-      <c r="H56" s="25"/>
-      <c r="I56" s="23" t="s">
+    <row r="57" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="H57" s="25"/>
+      <c r="I57" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="58" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="H58" s="25"/>
+      <c r="I58" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="57" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G57" s="23"/>
-      <c r="H57" s="25"/>
-      <c r="I57" s="23" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="58" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G58" s="23"/>
-      <c r="H58" s="25"/>
-      <c r="I58" s="23" t="s">
+    <row r="59" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="H59" s="25"/>
+      <c r="I59" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="60" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="H60" s="25"/>
+      <c r="I60" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="59" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G59" s="23"/>
-      <c r="H59" s="25"/>
-      <c r="I59" s="23" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="60" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G60" s="23"/>
-      <c r="H60" s="25"/>
-      <c r="I60" s="23" t="s">
-        <v>176</v>
-      </c>
-    </row>
     <row r="61" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G61" s="23" t="s">
+      <c r="G61" t="s">
         <v>36</v>
       </c>
       <c r="H61" s="24" t="s">
         <v>107</v>
       </c>
-      <c r="I61" s="23" t="s">
+      <c r="I61" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="62" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="G62" t="s">
+        <v>38</v>
+      </c>
+      <c r="H62" s="24"/>
+      <c r="I62" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="62" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G62" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="H62" s="24"/>
-      <c r="I62" s="23" t="s">
+    <row r="63" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="H63" s="24"/>
+      <c r="I63" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="64" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="H64" s="24"/>
+      <c r="I64" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="63" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G63" s="23"/>
-      <c r="H63" s="24"/>
-      <c r="I63" s="23" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="64" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G64" s="23"/>
-      <c r="H64" s="24"/>
-      <c r="I64" s="23" t="s">
-        <v>179</v>
-      </c>
-    </row>
     <row r="65" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G65" s="23"/>
       <c r="H65" s="24"/>
-      <c r="I65" s="23" t="s">
+      <c r="I65" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="66" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G66" s="23" t="s">
-        <v>177</v>
-      </c>
-      <c r="H66" s="26" t="s">
+      <c r="G66" t="s">
+        <v>176</v>
+      </c>
+      <c r="H66" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="I66" s="23" t="s">
+      <c r="I66" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="67" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G67" s="23" t="s">
+      <c r="G67" t="s">
         <v>12</v>
       </c>
       <c r="H67" s="25" t="s">
         <v>108</v>
       </c>
-      <c r="I67" s="23" t="s">
+      <c r="I67" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="68" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="H68" s="25"/>
+      <c r="I68" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="68" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G68" s="23"/>
-      <c r="H68" s="25"/>
-      <c r="I68" s="23" t="s">
-        <v>181</v>
-      </c>
-    </row>
     <row r="69" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G69" s="23" t="s">
+      <c r="G69" t="s">
         <v>18</v>
       </c>
       <c r="H69" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="I69" s="23" t="s">
+      <c r="I69" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="70" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G70" s="23" t="s">
-        <v>180</v>
+      <c r="G70" t="s">
+        <v>179</v>
       </c>
       <c r="H70" s="24"/>
-      <c r="I70" s="23" t="s">
+      <c r="I70" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="71" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G71" s="23"/>
       <c r="H71" s="24"/>
-      <c r="I71" s="23" t="s">
+      <c r="I71" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="72" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G72" s="23"/>
       <c r="H72" s="24"/>
-      <c r="I72" s="23" t="s">
+      <c r="I72" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="73" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G73" s="23"/>
       <c r="H73" s="24"/>
-      <c r="I73" s="23" t="s">
+      <c r="I73" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="74" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G74" s="23"/>
       <c r="H74" s="24"/>
-      <c r="I74" s="23" t="s">
+      <c r="I74" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="75" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G75" s="23"/>
       <c r="H75" s="24"/>
-      <c r="I75" s="23" t="s">
+      <c r="I75" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="76" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G76" s="23" t="s">
+      <c r="G76" t="s">
         <v>32</v>
       </c>
       <c r="H76" s="24" t="s">
         <v>109</v>
       </c>
-      <c r="I76" s="23" t="s">
+      <c r="I76" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="77" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G77" s="23"/>
       <c r="H77" s="24"/>
-      <c r="I77" s="23" t="s">
-        <v>182</v>
+      <c r="I77" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="78" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G78" s="23"/>
       <c r="H78" s="24"/>
-      <c r="I78" s="23" t="s">
+      <c r="I78" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="79" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G79" s="23"/>
       <c r="H79" s="24"/>
-      <c r="I79" s="23" t="s">
+      <c r="I79" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="80" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G80" s="23"/>
       <c r="H80" s="24"/>
-      <c r="I80" s="23" t="s">
+      <c r="I80" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="81" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G81" s="23"/>
       <c r="H81" s="24"/>
-      <c r="I81" s="23" t="s">
+      <c r="I81" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="82" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G82" s="23" t="s">
+      <c r="G82" t="s">
         <v>32</v>
       </c>
       <c r="H82" s="25" t="s">
         <v>110</v>
       </c>
-      <c r="I82" s="23" t="s">
+      <c r="I82" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="83" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G83" s="23" t="s">
+      <c r="G83" t="s">
         <v>75</v>
       </c>
       <c r="H83" s="25"/>
-      <c r="I83" s="23" t="s">
+      <c r="I83" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="84" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G84" s="23"/>
       <c r="H84" s="25"/>
-      <c r="I84" s="23" t="s">
+      <c r="I84" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="85" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G85" s="23"/>
       <c r="H85" s="25"/>
-      <c r="I85" s="23" t="s">
+      <c r="I85" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="86" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G86" s="23"/>
       <c r="H86" s="24" t="s">
         <v>111</v>
       </c>
-      <c r="I86" s="23" t="s">
+      <c r="I86" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="87" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="H87" s="24"/>
+      <c r="I87" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="87" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G87" s="23"/>
-      <c r="H87" s="24"/>
-      <c r="I87" s="23" t="s">
+    <row r="88" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="H88" s="24"/>
+      <c r="I88" t="s">
         <v>184</v>
-      </c>
-    </row>
-    <row r="88" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G88" s="23"/>
-      <c r="H88" s="24"/>
-      <c r="I88" s="23" t="s">
-        <v>185</v>
       </c>
     </row>
   </sheetData>
@@ -2163,22 +2118,22 @@
         <v>96</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="C2" s="16" t="s">
         <v>290</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="D2" s="20" t="s">
         <v>291</v>
       </c>
-      <c r="D2" s="20" t="s">
+      <c r="E2" s="17" t="s">
         <v>292</v>
       </c>
-      <c r="E2" s="17" t="s">
-        <v>293</v>
-      </c>
       <c r="F2" s="17" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="H2" s="5"/>
       <c r="I2" s="5"/>
@@ -2222,7 +2177,7 @@
         <v>1</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E4" s="17" t="s">
         <v>31</v>
@@ -2250,7 +2205,7 @@
         <v>33</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E5" s="17" t="s">
         <v>34</v>
@@ -2278,16 +2233,16 @@
         <v>1</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
@@ -2306,16 +2261,16 @@
         <v>1</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H7" s="5"/>
       <c r="I7" s="5"/>
@@ -2328,22 +2283,22 @@
         <v>97</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="H8" s="5"/>
       <c r="I8" s="5"/>
@@ -2356,22 +2311,22 @@
         <v>97</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C9" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F9" s="17" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G9" s="17" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
@@ -2384,22 +2339,22 @@
         <v>97</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C10" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F10" s="17" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="H10" s="5"/>
       <c r="I10" s="5"/>
@@ -2412,22 +2367,22 @@
         <v>97</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C11" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F11" s="17" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G11" s="17" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="H11" s="5"/>
       <c r="I11" s="5"/>
@@ -2440,22 +2395,22 @@
         <v>97</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C12" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="F12" s="17" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="G12" s="17" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="H12" s="5"/>
       <c r="I12" s="5"/>
@@ -2468,22 +2423,22 @@
         <v>97</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C13" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="F13" s="17" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="G13" s="17" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="H13" s="5"/>
       <c r="I13" s="5"/>
@@ -2496,13 +2451,13 @@
         <v>95</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E14" s="17" t="s">
         <v>37</v>
@@ -2524,13 +2479,13 @@
         <v>95</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C15" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E15" s="17" t="s">
         <v>39</v>
@@ -2558,7 +2513,7 @@
         <v>5</v>
       </c>
       <c r="D16" s="20" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E16" s="17" t="s">
         <v>41</v>
@@ -2586,7 +2541,7 @@
         <v>5</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E17" s="17" t="s">
         <v>43</v>
@@ -2608,13 +2563,13 @@
         <v>95</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C18" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D18" s="20" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E18" s="17" t="s">
         <v>45</v>
@@ -2636,13 +2591,13 @@
         <v>95</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C19" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E19" s="17" t="s">
         <v>47</v>
@@ -2664,13 +2619,13 @@
         <v>95</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C20" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D20" s="20" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E20" s="17" t="s">
         <v>48</v>
@@ -2692,13 +2647,13 @@
         <v>95</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C21" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D21" s="20" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E21" s="17" t="s">
         <v>49</v>
@@ -2720,13 +2675,13 @@
         <v>95</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C22" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D22" s="20" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E22" s="17" t="s">
         <v>51</v>
@@ -2748,13 +2703,13 @@
         <v>95</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C23" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E23" s="17" t="s">
         <v>52</v>
@@ -2776,13 +2731,13 @@
         <v>95</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C24" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D24" s="20" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E24" s="17" t="s">
         <v>54</v>
@@ -2804,13 +2759,13 @@
         <v>95</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C25" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D25" s="20" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E25" s="17" t="s">
         <v>55</v>
@@ -2832,13 +2787,13 @@
         <v>94</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C26" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D26" s="20" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E26" s="17" t="s">
         <v>56</v>
@@ -2860,13 +2815,13 @@
         <v>94</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C27" s="16" t="s">
         <v>5</v>
       </c>
       <c r="D27" s="20" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E27" s="17" t="s">
         <v>57</v>
@@ -2892,16 +2847,16 @@
       </c>
       <c r="C28" s="16"/>
       <c r="D28" s="20" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E28" s="17" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F28" s="17" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="G28" s="17" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="H28" s="17"/>
       <c r="I28" s="5"/>
@@ -2914,11 +2869,11 @@
         <v>94</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C29" s="16"/>
       <c r="D29" s="20" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E29" s="17" t="s">
         <v>35</v>
@@ -2946,7 +2901,7 @@
         <v>4</v>
       </c>
       <c r="D30" s="20" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E30" s="17" t="s">
         <v>58</v>
@@ -2974,16 +2929,16 @@
         <v>63</v>
       </c>
       <c r="D31" s="20" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E31" s="19" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F31" s="19" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G31" s="19" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="H31" s="5"/>
       <c r="I31" s="5"/>
@@ -2996,22 +2951,22 @@
         <v>93</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C32" s="16" t="s">
         <v>63</v>
       </c>
       <c r="D32" s="20" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E32" s="19" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F32" s="19" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="G32" s="19" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="H32" s="5"/>
       <c r="I32" s="5"/>
@@ -3024,22 +2979,22 @@
         <v>93</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C33" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D33" s="20" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E33" s="17" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F33" s="17" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G33" s="17" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="H33" s="5"/>
       <c r="I33" s="5"/>
@@ -3058,7 +3013,7 @@
         <v>59</v>
       </c>
       <c r="D34" s="20" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="E34" s="17" t="s">
         <v>60</v>
@@ -3086,16 +3041,16 @@
         <v>98</v>
       </c>
       <c r="D35" s="20" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="E35" s="17" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F35" s="17" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="G35" s="17" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="H35" s="5"/>
       <c r="I35" s="5"/>
@@ -3111,19 +3066,19 @@
         <v>22</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D36" s="20" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E36" s="17" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F36" s="17" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="G36" s="17" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="H36" s="5"/>
       <c r="I36" s="5"/>
@@ -3142,16 +3097,16 @@
         <v>63</v>
       </c>
       <c r="D37" s="20" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E37" s="17" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F37" s="17" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="G37" s="17" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H37" s="5"/>
       <c r="I37" s="5"/>
@@ -3170,7 +3125,7 @@
         <v>63</v>
       </c>
       <c r="D38" s="20" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E38" s="17" t="s">
         <v>64</v>
@@ -3198,7 +3153,7 @@
         <v>63</v>
       </c>
       <c r="D39" s="20" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E39" s="17" t="s">
         <v>66</v>
@@ -3226,16 +3181,16 @@
         <v>63</v>
       </c>
       <c r="D40" s="20" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E40" s="17" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F40" s="17" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G40" s="17" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="H40" s="17"/>
       <c r="I40" s="5"/>
@@ -3248,13 +3203,13 @@
         <v>90</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C41" s="16" t="s">
         <v>69</v>
       </c>
       <c r="D41" s="20" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E41" s="17" t="s">
         <v>70</v>
@@ -3276,13 +3231,13 @@
         <v>90</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C42" s="16" t="s">
         <v>71</v>
       </c>
       <c r="D42" s="20" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E42" s="17" t="s">
         <v>72</v>
@@ -3304,22 +3259,22 @@
         <v>90</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C43" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D43" s="20" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E43" s="17" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="H43" s="5"/>
       <c r="I43" s="5"/>
@@ -3338,16 +3293,16 @@
         <v>4</v>
       </c>
       <c r="D44" s="20" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E44" s="17" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="H44" s="5"/>
       <c r="I44" s="5"/>
@@ -3366,7 +3321,7 @@
         <v>1</v>
       </c>
       <c r="D45" s="20" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E45" s="17" t="s">
         <v>76</v>
@@ -3394,16 +3349,16 @@
         <v>33</v>
       </c>
       <c r="D46" s="20" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E46" s="17" t="s">
         <v>78</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G46" s="5" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="H46" s="5"/>
       <c r="I46" s="5"/>
@@ -3422,7 +3377,7 @@
         <v>69</v>
       </c>
       <c r="D47" s="20" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E47" s="17" t="s">
         <v>80</v>
@@ -3450,7 +3405,7 @@
         <v>69</v>
       </c>
       <c r="D48" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E48" s="17" t="s">
         <v>82</v>
@@ -3478,7 +3433,7 @@
         <v>4</v>
       </c>
       <c r="D49" s="20" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E49" s="17" t="s">
         <v>84</v>
@@ -3506,16 +3461,16 @@
         <v>4</v>
       </c>
       <c r="D50" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E50" s="17" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F50" s="17" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="G50" s="17" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="H50" s="5"/>
       <c r="I50" s="5"/>
@@ -3528,22 +3483,22 @@
         <v>111</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C51" s="16" t="s">
         <v>69</v>
       </c>
       <c r="D51" s="20" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E51" s="19" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F51" s="19" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="G51" s="19" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="H51" s="5"/>
       <c r="I51" s="5"/>
@@ -3556,22 +3511,22 @@
         <v>111</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C52" s="16" t="s">
         <v>71</v>
       </c>
       <c r="D52" s="20" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E52" s="19" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F52" s="19" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G52" s="19" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="H52" s="5"/>
       <c r="I52" s="5"/>
@@ -4342,7 +4297,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E71F352-39EA-49E2-AB89-A39562B80CB1}">
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.109375" bestFit="1" customWidth="1"/>
@@ -4428,22 +4383,22 @@
         <v>95</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>3</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="H5" s="5"/>
       <c r="I5" s="5"/>
@@ -4453,13 +4408,13 @@
         <v>95</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>3</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>112</v>
@@ -4484,16 +4439,16 @@
         <v>4</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="H7" s="5"/>
       <c r="I7" s="5"/>
@@ -4503,22 +4458,22 @@
         <v>95</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>4</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H8" s="5"/>
       <c r="I8" s="5"/>
@@ -4528,22 +4483,22 @@
         <v>95</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>114</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
@@ -4553,22 +4508,22 @@
         <v>95</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>3</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H10" s="5"/>
       <c r="I10" s="5"/>
@@ -4578,22 +4533,22 @@
         <v>95</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>71</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H11" s="5"/>
       <c r="I11" s="5"/>
@@ -4603,22 +4558,22 @@
         <v>95</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>114</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H12" s="5"/>
       <c r="I12" s="5"/>
@@ -4628,22 +4583,22 @@
         <v>95</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>3</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="H13" s="5"/>
       <c r="I13" s="5"/>
@@ -4653,22 +4608,22 @@
         <v>95</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>71</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H14" s="5"/>
       <c r="I14" s="5"/>
@@ -4678,22 +4633,22 @@
         <v>95</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>114</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
@@ -4703,22 +4658,22 @@
         <v>95</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>3</v>
       </c>
       <c r="D16" s="21" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="H16" s="5"/>
       <c r="I16" s="5"/>
@@ -4741,20 +4696,20 @@
         <v>99</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="21" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="H18" s="5"/>
       <c r="I18" s="5"/>
@@ -4777,20 +4732,20 @@
         <v>92</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="21" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="H20" s="5"/>
       <c r="I20" s="5"/>
@@ -4800,20 +4755,20 @@
         <v>92</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>115</v>
+        <v>322</v>
       </c>
       <c r="C21" s="6"/>
       <c r="D21" s="21" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H21" s="5"/>
       <c r="I21" s="5"/>
@@ -4823,20 +4778,22 @@
         <v>92</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="C22" s="6"/>
+        <v>115</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>323</v>
+      </c>
       <c r="D22" s="21" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="H22" s="5"/>
       <c r="I22" s="5"/>
@@ -4849,94 +4806,92 @@
         <v>13</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D23" s="21" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H23" s="5"/>
       <c r="I23" s="5"/>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A24" s="18" t="s">
-        <v>92</v>
+      <c r="A24" s="15" t="s">
+        <v>90</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>4</v>
-      </c>
+        <v>123</v>
+      </c>
+      <c r="C24" s="6"/>
       <c r="D24" s="21" t="s">
-        <v>287</v>
+        <v>268</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>149</v>
+        <v>245</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>149</v>
+        <v>125</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>149</v>
+        <v>125</v>
       </c>
       <c r="H24" s="5"/>
       <c r="I24" s="5"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A25" s="18" t="s">
-        <v>92</v>
+      <c r="A25" s="15" t="s">
+        <v>90</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D25" s="21" t="s">
-        <v>288</v>
+        <v>269</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>150</v>
+        <v>126</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>150</v>
+        <v>126</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>150</v>
+        <v>126</v>
       </c>
       <c r="H25" s="5"/>
       <c r="I25" s="5"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A26" s="18" t="s">
-        <v>92</v>
+      <c r="A26" s="15" t="s">
+        <v>90</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>120</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="D26" s="21" t="s">
-        <v>289</v>
+        <v>278</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>151</v>
+        <v>246</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>151</v>
+        <v>247</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>151</v>
+        <v>247</v>
       </c>
       <c r="H26" s="5"/>
       <c r="I26" s="5"/>
@@ -4946,95 +4901,97 @@
         <v>90</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="C27" s="6"/>
+        <v>121</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>1</v>
+      </c>
       <c r="D27" s="21" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>246</v>
+        <v>127</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H27" s="5"/>
       <c r="I27" s="5"/>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A28" s="15" t="s">
-        <v>90</v>
+      <c r="A28" s="18" t="s">
+        <v>91</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>1</v>
+        <v>69</v>
       </c>
       <c r="D28" s="21" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="H28" s="5"/>
       <c r="I28" s="5"/>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A29" s="15" t="s">
-        <v>90</v>
+      <c r="A29" s="18" t="s">
+        <v>91</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>125</v>
+        <v>69</v>
       </c>
       <c r="D29" s="21" t="s">
-        <v>279</v>
+        <v>261</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>247</v>
+        <v>137</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>248</v>
+        <v>137</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>248</v>
+        <v>137</v>
       </c>
       <c r="H29" s="5"/>
       <c r="I29" s="5"/>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A30" s="15" t="s">
-        <v>90</v>
+      <c r="A30" s="18" t="s">
+        <v>91</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="C30" s="6" t="s">
         <v>1</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="H30" s="5"/>
       <c r="I30" s="5"/>
@@ -5047,19 +5004,19 @@
         <v>129</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>69</v>
+        <v>33</v>
       </c>
       <c r="D31" s="21" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H31" s="5"/>
       <c r="I31" s="5"/>
@@ -5069,22 +5026,22 @@
         <v>91</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C32" s="6" t="s">
         <v>69</v>
       </c>
       <c r="D32" s="21" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="H32" s="5"/>
       <c r="I32" s="5"/>
@@ -5094,22 +5051,22 @@
         <v>91</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>1</v>
+        <v>69</v>
       </c>
       <c r="D33" s="21" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="H33" s="5"/>
       <c r="I33" s="5"/>
@@ -5119,131 +5076,141 @@
         <v>91</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="D34" s="21" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="H34" s="5"/>
-      <c r="I34" s="5"/>
+        <v>142</v>
+      </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" s="18" t="s">
         <v>91</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>69</v>
+        <v>33</v>
       </c>
       <c r="D35" s="21" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="H35" s="5"/>
-      <c r="I35" s="5"/>
+        <v>143</v>
+      </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A36" s="18" t="s">
-        <v>91</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="C36" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="D36" s="21" t="s">
-        <v>266</v>
-      </c>
-      <c r="E36" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="F36" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="G36" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="H36" s="5"/>
-      <c r="I36" s="5"/>
+      <c r="B36" s="7"/>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A37" s="18" t="s">
-        <v>91</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="D37" s="21" t="s">
-        <v>267</v>
-      </c>
-      <c r="E37" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="F37" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="G37" s="5" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A38" s="18" t="s">
-        <v>91</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="C38" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="D38" s="21" t="s">
-        <v>268</v>
-      </c>
-      <c r="E38" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="F38" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="G38" s="5" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B39" s="7"/>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B40" s="7"/>
+      <c r="B37" s="7"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6C1B83A-C39F-40B8-8309-44C0020910F4}">
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="21" t="s">
+        <v>286</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="21" t="s">
+        <v>287</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="D3" s="21" t="s">
+        <v>288</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update RCA workbook metadata
</commit_message>
<xml_diff>
--- a/eBus_Functions/Post_Processing/Root_Cause_Analysis_Work/info/eBus_Model_Info.xlsx
+++ b/eBus_Functions/Post_Processing/Root_Cause_Analysis_Work/info/eBus_Model_Info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TempData\Github\eBus_Tool\eBus_Functions\Post_Processing\Root_Cause_Analysis_Work\info\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8325D24C-37B5-484E-BEFB-0DD5230CE88D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6579860E-F8BB-4EE3-915C-DF903BFDBA69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Block_Diagram" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="324">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="701" uniqueCount="332">
   <si>
     <t>Driver</t>
   </si>
@@ -582,9 +582,6 @@
     <t>Auxiliary Load Voltage</t>
   </si>
   <si>
-    <t>Auxiliary Load Power</t>
-  </si>
-  <si>
     <t>logout.CmdTrq_Req_PTIce1/2</t>
   </si>
   <si>
@@ -729,15 +726,6 @@
     <t>logout.pne_brk_Axle1_BrakingPower+logout.pne_brk_Axle2_BrakingPower+logout.pne_brk_Axle3_BrakingPower+logout.pne_brk_Axle4_BrakingPower</t>
   </si>
   <si>
-    <t>logout.hvs_zfCetrax_gbxOut_torque*sMP.global.mec_iDiffAxle/(sMP.global.mec_rWheelDriven*0.001)-(logout.mec_brk_Axle1_TiBrk_info+logout.mec_brk_Axle2_TiBrk_info+logout.mec_brk_Axle3_TiBrk_info+logout.mec_brk_Axle4_TiBrk_info)</t>
-  </si>
-  <si>
-    <t>logout.mec_brk_Axle1_TiBrk_info+logout.mec_brk_Axle2_TiBrk_info+logout.mec_brk_Axle3_TiBrk_info+logout.mec_brk_Axle4_TiBrk_info</t>
-  </si>
-  <si>
-    <t>logout.mec_brk_Wheel1_TiLossRollRes_info+logout.mec_brk_Wheel2_TiLossRollRes_info+logout.mec_brk_Wheel3_TiLossRollRes_info+logout.mec_brk_Wheel4_TiLossRollRes_info</t>
-  </si>
-  <si>
     <t>logout.eess_BatHW_P_BatPwr/1000</t>
   </si>
   <si>
@@ -1000,6 +988,46 @@
   </si>
   <si>
     <t>m</t>
+  </si>
+  <si>
+    <t>Inertial Force</t>
+  </si>
+  <si>
+    <t>veh_ma</t>
+  </si>
+  <si>
+    <t>logout.mec_veh_transAcc*sMP.global.mec_massVehicle_kg</t>
+  </si>
+  <si>
+    <t>(logout.mec_brk_Wheel1_TiLossRollRes_info+logout.mec_brk_Wheel2_TiLossRollRes_info+logout.mec_brk_Wheel3_TiLossRollRes_info+logout.mec_brk_Wheel4_TiLossRollRes_info)/(sMP.global.mec_rWheelDriven*0.001)</t>
+  </si>
+  <si>
+    <t>veh_long_force</t>
+  </si>
+  <si>
+    <t>logout.hvs_zfCetrax_gbxOut_torque*sMP.global.mec_iDiffAxle/(sMP.global.mec_rWheelDriven*0.001)</t>
+  </si>
+  <si>
+    <t>logout.hvs_zfCetrax_gbxOut_torque*sMP.global.mec_iDiffAxle</t>
+  </si>
+  <si>
+    <t>Vehicle Propulsion Force</t>
+  </si>
+  <si>
+    <t>(logout.mec_brk_Axle1_TiBrk_info+logout.mec_brk_Axle2_TiBrk_info+logout.mec_brk_Axle3_TiBrk_info+logout.mec_brk_Axle4_TiBrk_info)//(sMP.global.mec_rWheelDriven*0.001)</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>These Battery Current and Power Limits are sent to Powertrain Controller, so that power train controller can demand the torque, that is adhered to these limits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In Vehicle Dynamics, 
+Vehicle Propulsion Force = Net Traction Torque / Tire Radius;
+Vehicle Propulsion Force - Friction Brake Force = Wheel Force;
+Wheel Force = AeroDynamic Force + Gradient Force + Rolling Resistance Force + Inertial Force;
+</t>
   </si>
 </sst>
 </file>
@@ -1120,7 +1148,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -1159,11 +1187,136 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1216,17 +1369,66 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1309,7 +1511,7 @@
       <xdr:col>8</xdr:col>
       <xdr:colOff>2972078</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>53340</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1608,16 +1810,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="G27:I88"/>
+  <dimension ref="G27:J88"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="7" max="7" width="30.109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="26.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="54" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="82.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="27" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="28" spans="7:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="7:10" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="28" spans="7:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G28" s="8" t="s">
         <v>8</v>
       </c>
@@ -1627,440 +1830,565 @@
       <c r="I28" s="10" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="29" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H29" s="24" t="s">
+      <c r="J28" s="9" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="29" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G29" s="22"/>
+      <c r="H29" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="I29" t="s">
+      <c r="I29" s="23" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="30" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H30" s="24"/>
-      <c r="I30" t="s">
+      <c r="J29" s="28"/>
+    </row>
+    <row r="30" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G30" s="24"/>
+      <c r="H30" s="38"/>
+      <c r="I30" s="25" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="31" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H31" s="24"/>
-      <c r="I31" t="s">
+      <c r="J30" s="29"/>
+    </row>
+    <row r="31" spans="7:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G31" s="26"/>
+      <c r="H31" s="39"/>
+      <c r="I31" s="27" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="32" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G32" t="s">
+      <c r="J31" s="30"/>
+    </row>
+    <row r="32" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G32" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="H32" s="25" t="s">
+      <c r="H32" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="I32" t="s">
+      <c r="I32" s="23" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="33" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G33" t="s">
+      <c r="J32" s="28"/>
+    </row>
+    <row r="33" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G33" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="H33" s="25"/>
-      <c r="I33" t="s">
+      <c r="H33" s="41"/>
+      <c r="I33" s="25" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="34" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G34" t="s">
+      <c r="J33" s="29"/>
+    </row>
+    <row r="34" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G34" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="H34" s="25"/>
-    </row>
-    <row r="35" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G35" t="s">
+      <c r="H34" s="41"/>
+      <c r="I34" s="25"/>
+      <c r="J34" s="29"/>
+    </row>
+    <row r="35" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G35" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="H35" s="25"/>
-    </row>
-    <row r="36" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G36" t="s">
+      <c r="H35" s="41"/>
+      <c r="I35" s="25"/>
+      <c r="J35" s="29"/>
+    </row>
+    <row r="36" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G36" s="24" t="s">
         <v>178</v>
       </c>
-      <c r="H36" s="25"/>
-    </row>
-    <row r="37" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G37" t="s">
+      <c r="H36" s="41"/>
+      <c r="I36" s="25"/>
+      <c r="J36" s="29"/>
+    </row>
+    <row r="37" spans="7:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G37" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="H37" s="25"/>
-    </row>
-    <row r="38" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G38" t="s">
+      <c r="H37" s="42"/>
+      <c r="I37" s="27"/>
+      <c r="J37" s="30"/>
+    </row>
+    <row r="38" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G38" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="H38" s="24" t="s">
+      <c r="H38" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="I38" t="s">
+      <c r="I38" s="23" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="39" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G39" t="s">
+      <c r="J38" s="28"/>
+    </row>
+    <row r="39" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G39" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="H39" s="24"/>
-      <c r="I39" t="s">
+      <c r="H39" s="38"/>
+      <c r="I39" s="25" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="40" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H40" s="24"/>
-      <c r="I40" t="s">
+      <c r="J39" s="29"/>
+    </row>
+    <row r="40" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G40" s="24"/>
+      <c r="H40" s="38"/>
+      <c r="I40" s="25" t="s">
+        <v>302</v>
+      </c>
+      <c r="J40" s="29"/>
+    </row>
+    <row r="41" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G41" s="24"/>
+      <c r="H41" s="38"/>
+      <c r="I41" s="25" t="s">
+        <v>303</v>
+      </c>
+      <c r="J41" s="29"/>
+    </row>
+    <row r="42" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G42" s="24"/>
+      <c r="H42" s="38"/>
+      <c r="I42" s="25" t="s">
         <v>306</v>
       </c>
-    </row>
-    <row r="41" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H41" s="24"/>
-      <c r="I41" t="s">
+      <c r="J42" s="29"/>
+    </row>
+    <row r="43" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G43" s="24"/>
+      <c r="H43" s="38"/>
+      <c r="I43" s="25" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="42" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H42" s="24"/>
-      <c r="I42" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="43" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H43" s="24"/>
-      <c r="I43" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="44" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H44" s="24"/>
-    </row>
-    <row r="45" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H45" s="24"/>
-    </row>
-    <row r="46" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H46" s="24"/>
-    </row>
-    <row r="47" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H47" s="24"/>
-    </row>
-    <row r="48" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H48" s="22"/>
-    </row>
-    <row r="49" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G49" t="s">
+      <c r="J43" s="29"/>
+    </row>
+    <row r="44" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G44" s="24"/>
+      <c r="H44" s="38"/>
+      <c r="I44" s="25"/>
+      <c r="J44" s="29"/>
+    </row>
+    <row r="45" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G45" s="24"/>
+      <c r="H45" s="38"/>
+      <c r="I45" s="25"/>
+      <c r="J45" s="29"/>
+    </row>
+    <row r="46" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G46" s="24"/>
+      <c r="H46" s="38"/>
+      <c r="I46" s="25"/>
+      <c r="J46" s="29"/>
+    </row>
+    <row r="47" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G47" s="24"/>
+      <c r="H47" s="38"/>
+      <c r="I47" s="25"/>
+      <c r="J47" s="29"/>
+    </row>
+    <row r="48" spans="7:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G48" s="26"/>
+      <c r="H48" s="39"/>
+      <c r="I48" s="27"/>
+      <c r="J48" s="30"/>
+    </row>
+    <row r="49" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G49" s="22" t="s">
         <v>170</v>
       </c>
-      <c r="H49" s="25" t="s">
+      <c r="H49" s="40" t="s">
         <v>106</v>
       </c>
-      <c r="I49" t="s">
+      <c r="I49" s="31" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="50" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G50" t="s">
+      <c r="J49" s="28"/>
+    </row>
+    <row r="50" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G50" s="24" t="s">
         <v>171</v>
       </c>
-      <c r="H50" s="25"/>
-      <c r="I50" t="s">
+      <c r="H50" s="41"/>
+      <c r="I50" s="32" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="51" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G51" t="s">
-        <v>308</v>
-      </c>
-      <c r="H51" s="25"/>
-      <c r="I51" t="s">
+      <c r="J50" s="29"/>
+    </row>
+    <row r="51" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G51" s="24" t="s">
+        <v>304</v>
+      </c>
+      <c r="H51" s="41"/>
+      <c r="I51" s="32" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="52" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G52" t="s">
-        <v>309</v>
-      </c>
-      <c r="H52" s="25"/>
-      <c r="I52" t="s">
+      <c r="J51" s="29"/>
+    </row>
+    <row r="52" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G52" s="24" t="s">
+        <v>305</v>
+      </c>
+      <c r="H52" s="41"/>
+      <c r="I52" s="32" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="53" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H53" s="25"/>
-      <c r="I53" t="s">
+      <c r="J52" s="29"/>
+    </row>
+    <row r="53" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G53" s="24"/>
+      <c r="H53" s="41"/>
+      <c r="I53" s="32" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="54" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H54" s="25"/>
-      <c r="I54" t="s">
+      <c r="J53" s="29"/>
+    </row>
+    <row r="54" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G54" s="24"/>
+      <c r="H54" s="41"/>
+      <c r="I54" s="32" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="55" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H55" s="25"/>
-      <c r="I55" t="s">
+      <c r="J54" s="29"/>
+    </row>
+    <row r="55" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G55" s="24"/>
+      <c r="H55" s="41"/>
+      <c r="I55" s="32" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="56" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H56" s="25"/>
-      <c r="I56" t="s">
+      <c r="J55" s="29"/>
+    </row>
+    <row r="56" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G56" s="24"/>
+      <c r="H56" s="41"/>
+      <c r="I56" s="32" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="57" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H57" s="25"/>
-      <c r="I57" t="s">
+      <c r="J56" s="29"/>
+    </row>
+    <row r="57" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G57" s="24"/>
+      <c r="H57" s="41"/>
+      <c r="I57" s="32" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="58" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H58" s="25"/>
-      <c r="I58" t="s">
+      <c r="J57" s="29"/>
+    </row>
+    <row r="58" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G58" s="24"/>
+      <c r="H58" s="41"/>
+      <c r="I58" s="32" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="59" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H59" s="25"/>
-      <c r="I59" t="s">
+      <c r="J58" s="29"/>
+    </row>
+    <row r="59" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G59" s="24"/>
+      <c r="H59" s="41"/>
+      <c r="I59" s="32" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="60" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H60" s="25"/>
-      <c r="I60" t="s">
+      <c r="J59" s="29"/>
+    </row>
+    <row r="60" spans="7:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G60" s="26"/>
+      <c r="H60" s="42"/>
+      <c r="I60" s="33" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="61" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G61" t="s">
+      <c r="J60" s="30"/>
+    </row>
+    <row r="61" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G61" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="H61" s="24" t="s">
+      <c r="H61" s="37" t="s">
         <v>107</v>
       </c>
-      <c r="I61" t="s">
+      <c r="I61" s="31" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="62" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G62" t="s">
+      <c r="J61" s="28"/>
+    </row>
+    <row r="62" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G62" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="H62" s="24"/>
-      <c r="I62" t="s">
+      <c r="H62" s="38"/>
+      <c r="I62" s="32" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="63" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H63" s="24"/>
-      <c r="I63" t="s">
+      <c r="J62" s="29"/>
+    </row>
+    <row r="63" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G63" s="24"/>
+      <c r="H63" s="38"/>
+      <c r="I63" s="32" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="64" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H64" s="24"/>
-      <c r="I64" t="s">
+      <c r="J63" s="29"/>
+    </row>
+    <row r="64" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G64" s="24"/>
+      <c r="H64" s="38"/>
+      <c r="I64" s="32" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="65" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H65" s="24"/>
-      <c r="I65" t="s">
+      <c r="J64" s="29"/>
+    </row>
+    <row r="65" spans="7:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G65" s="26"/>
+      <c r="H65" s="39"/>
+      <c r="I65" s="33" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="66" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G66" t="s">
+      <c r="J65" s="30"/>
+    </row>
+    <row r="66" spans="7:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G66" s="34" t="s">
         <v>176</v>
       </c>
-      <c r="H66" s="23" t="s">
+      <c r="H66" s="43" t="s">
         <v>17</v>
       </c>
-      <c r="I66" t="s">
+      <c r="I66" s="35" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="67" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G67" t="s">
+      <c r="J66" s="36"/>
+    </row>
+    <row r="67" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G67" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="H67" s="25" t="s">
+      <c r="H67" s="40" t="s">
         <v>108</v>
       </c>
-      <c r="I67" t="s">
+      <c r="I67" s="31" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="68" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H68" s="25"/>
-      <c r="I68" t="s">
+      <c r="J67" s="28"/>
+    </row>
+    <row r="68" spans="7:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G68" s="26"/>
+      <c r="H68" s="42"/>
+      <c r="I68" s="33" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="69" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G69" t="s">
-        <v>18</v>
-      </c>
-      <c r="H69" s="24" t="s">
+      <c r="J68" s="30"/>
+    </row>
+    <row r="69" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G69" s="22" t="s">
+        <v>327</v>
+      </c>
+      <c r="H69" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="I69" t="s">
+      <c r="I69" s="31" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="70" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G70" t="s">
+      <c r="J69" s="48" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="70" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G70" s="24" t="s">
         <v>179</v>
       </c>
-      <c r="H70" s="24"/>
-      <c r="I70" t="s">
+      <c r="H70" s="38"/>
+      <c r="I70" s="32" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="71" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H71" s="24"/>
-      <c r="I71" t="s">
+      <c r="J70" s="49"/>
+    </row>
+    <row r="71" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G71" s="24"/>
+      <c r="H71" s="38"/>
+      <c r="I71" s="32" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="72" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H72" s="24"/>
-      <c r="I72" t="s">
+      <c r="J71" s="49"/>
+    </row>
+    <row r="72" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G72" s="24"/>
+      <c r="H72" s="38"/>
+      <c r="I72" s="32" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="73" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H73" s="24"/>
-      <c r="I73" t="s">
+      <c r="J72" s="49"/>
+    </row>
+    <row r="73" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G73" s="24"/>
+      <c r="H73" s="38"/>
+      <c r="I73" s="32" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="74" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H74" s="24"/>
-      <c r="I74" t="s">
+      <c r="J73" s="49"/>
+    </row>
+    <row r="74" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G74" s="24"/>
+      <c r="H74" s="38"/>
+      <c r="I74" s="32" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="75" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H75" s="24"/>
-      <c r="I75" t="s">
+      <c r="J74" s="49"/>
+    </row>
+    <row r="75" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G75" s="24"/>
+      <c r="H75" s="38"/>
+      <c r="I75" s="44" t="s">
+        <v>320</v>
+      </c>
+      <c r="J75" s="49"/>
+    </row>
+    <row r="76" spans="7:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G76" s="26"/>
+      <c r="H76" s="39"/>
+      <c r="I76" s="33" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="76" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G76" t="s">
+      <c r="J76" s="50"/>
+    </row>
+    <row r="77" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G77" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="H76" s="24" t="s">
+      <c r="H77" s="37" t="s">
         <v>109</v>
       </c>
-      <c r="I76" t="s">
+      <c r="I77" s="31" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="77" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H77" s="24"/>
-      <c r="I77" t="s">
+      <c r="J77" s="45"/>
+    </row>
+    <row r="78" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G78" s="24"/>
+      <c r="H78" s="38"/>
+      <c r="I78" s="32" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="78" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H78" s="24"/>
-      <c r="I78" t="s">
+      <c r="J78" s="46"/>
+    </row>
+    <row r="79" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G79" s="24"/>
+      <c r="H79" s="38"/>
+      <c r="I79" s="32" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="79" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H79" s="24"/>
-      <c r="I79" t="s">
+      <c r="J79" s="46"/>
+    </row>
+    <row r="80" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G80" s="24"/>
+      <c r="H80" s="38"/>
+      <c r="I80" s="32" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="80" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H80" s="24"/>
-      <c r="I80" t="s">
+      <c r="J80" s="46"/>
+    </row>
+    <row r="81" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G81" s="24"/>
+      <c r="H81" s="38"/>
+      <c r="I81" s="32" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="81" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H81" s="24"/>
-      <c r="I81" t="s">
+      <c r="J81" s="46"/>
+    </row>
+    <row r="82" spans="7:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G82" s="26"/>
+      <c r="H82" s="39"/>
+      <c r="I82" s="33" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="82" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G82" t="s">
+      <c r="J82" s="47"/>
+    </row>
+    <row r="83" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G83" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="H82" s="25" t="s">
+      <c r="H83" s="40" t="s">
         <v>110</v>
       </c>
-      <c r="I82" t="s">
+      <c r="I83" s="31" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="83" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G83" t="s">
+      <c r="J83" s="48" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="84" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G84" s="24" t="s">
         <v>75</v>
       </c>
-      <c r="H83" s="25"/>
-      <c r="I83" t="s">
+      <c r="H84" s="41"/>
+      <c r="I84" s="32" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="84" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H84" s="25"/>
-      <c r="I84" t="s">
+      <c r="J84" s="49"/>
+    </row>
+    <row r="85" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G85" s="24"/>
+      <c r="H85" s="41"/>
+      <c r="I85" s="32" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="85" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H85" s="25"/>
-      <c r="I85" t="s">
+      <c r="J85" s="49"/>
+    </row>
+    <row r="86" spans="7:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G86" s="26"/>
+      <c r="H86" s="42"/>
+      <c r="I86" s="33" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="86" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H86" s="24" t="s">
+      <c r="J86" s="50"/>
+    </row>
+    <row r="87" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G87" s="22"/>
+      <c r="H87" s="37" t="s">
         <v>111</v>
       </c>
-      <c r="I86" t="s">
+      <c r="I87" s="31" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="87" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H87" s="24"/>
-      <c r="I87" t="s">
+      <c r="J87" s="28"/>
+    </row>
+    <row r="88" spans="7:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G88" s="26"/>
+      <c r="H88" s="39"/>
+      <c r="I88" s="33" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="88" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="H88" s="24"/>
-      <c r="I88" t="s">
-        <v>184</v>
-      </c>
+      <c r="J88" s="30"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="20">
+    <mergeCell ref="J87:J88"/>
+    <mergeCell ref="J77:J82"/>
+    <mergeCell ref="J69:J76"/>
+    <mergeCell ref="J67:J68"/>
+    <mergeCell ref="H38:H48"/>
+    <mergeCell ref="J83:J86"/>
+    <mergeCell ref="J29:J31"/>
+    <mergeCell ref="J32:J37"/>
+    <mergeCell ref="J38:J48"/>
+    <mergeCell ref="J49:J60"/>
+    <mergeCell ref="J61:J65"/>
+    <mergeCell ref="H77:H82"/>
+    <mergeCell ref="H83:H86"/>
+    <mergeCell ref="H61:H65"/>
+    <mergeCell ref="H69:H76"/>
+    <mergeCell ref="H87:H88"/>
     <mergeCell ref="H29:H31"/>
     <mergeCell ref="H32:H37"/>
-    <mergeCell ref="H38:H47"/>
     <mergeCell ref="H49:H60"/>
     <mergeCell ref="H67:H68"/>
-    <mergeCell ref="H76:H81"/>
-    <mergeCell ref="H82:H85"/>
-    <mergeCell ref="H61:H65"/>
-    <mergeCell ref="H69:H75"/>
-    <mergeCell ref="H86:H88"/>
   </mergeCells>
   <conditionalFormatting sqref="I29:I88 G29:G88">
-    <cfRule type="duplicateValues" dxfId="4" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="13"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2070,7 +2398,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFA16316-83DB-41C7-8B25-B191695DD108}">
-  <dimension ref="A1:L105"/>
+  <dimension ref="A1:L107"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.109375" bestFit="1" customWidth="1"/>
@@ -2118,22 +2446,22 @@
         <v>96</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="H2" s="5"/>
       <c r="I2" s="5"/>
@@ -2177,7 +2505,7 @@
         <v>1</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E4" s="17" t="s">
         <v>31</v>
@@ -2205,7 +2533,7 @@
         <v>33</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E5" s="17" t="s">
         <v>34</v>
@@ -2233,16 +2561,16 @@
         <v>1</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
@@ -2261,16 +2589,16 @@
         <v>1</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="H7" s="5"/>
       <c r="I7" s="5"/>
@@ -2283,22 +2611,22 @@
         <v>97</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="H8" s="5"/>
       <c r="I8" s="5"/>
@@ -2311,22 +2639,22 @@
         <v>97</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="C9" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F9" s="17" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G9" s="17" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
@@ -2339,22 +2667,22 @@
         <v>97</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="C10" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D10" s="20" t="s">
+        <v>312</v>
+      </c>
+      <c r="E10" s="17" t="s">
         <v>316</v>
       </c>
-      <c r="E10" s="17" t="s">
-        <v>320</v>
-      </c>
       <c r="F10" s="17" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="H10" s="5"/>
       <c r="I10" s="5"/>
@@ -2367,22 +2695,22 @@
         <v>97</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="C11" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="F11" s="17" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="G11" s="17" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="H11" s="5"/>
       <c r="I11" s="5"/>
@@ -2395,22 +2723,22 @@
         <v>97</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="C12" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="F12" s="17" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="G12" s="17" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="H12" s="5"/>
       <c r="I12" s="5"/>
@@ -2423,22 +2751,22 @@
         <v>97</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="C13" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="F13" s="17" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="G13" s="17" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="H13" s="5"/>
       <c r="I13" s="5"/>
@@ -2451,13 +2779,13 @@
         <v>95</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E14" s="17" t="s">
         <v>37</v>
@@ -2479,13 +2807,13 @@
         <v>95</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="C15" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E15" s="17" t="s">
         <v>39</v>
@@ -2513,7 +2841,7 @@
         <v>5</v>
       </c>
       <c r="D16" s="20" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E16" s="17" t="s">
         <v>41</v>
@@ -2541,7 +2869,7 @@
         <v>5</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E17" s="17" t="s">
         <v>43</v>
@@ -2563,13 +2891,13 @@
         <v>95</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="C18" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D18" s="20" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E18" s="17" t="s">
         <v>45</v>
@@ -2591,13 +2919,13 @@
         <v>95</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="C19" s="16" t="s">
         <v>4</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E19" s="17" t="s">
         <v>47</v>
@@ -2625,7 +2953,7 @@
         <v>4</v>
       </c>
       <c r="D20" s="20" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E20" s="17" t="s">
         <v>48</v>
@@ -2653,7 +2981,7 @@
         <v>4</v>
       </c>
       <c r="D21" s="20" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E21" s="17" t="s">
         <v>49</v>
@@ -2675,13 +3003,13 @@
         <v>95</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="C22" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D22" s="20" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E22" s="17" t="s">
         <v>51</v>
@@ -2703,13 +3031,13 @@
         <v>95</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="C23" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E23" s="17" t="s">
         <v>52</v>
@@ -2731,13 +3059,13 @@
         <v>95</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="C24" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D24" s="20" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E24" s="17" t="s">
         <v>54</v>
@@ -2759,13 +3087,13 @@
         <v>95</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="C25" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D25" s="20" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E25" s="17" t="s">
         <v>55</v>
@@ -2787,13 +3115,13 @@
         <v>94</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="C26" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D26" s="20" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E26" s="17" t="s">
         <v>56</v>
@@ -2821,7 +3149,7 @@
         <v>5</v>
       </c>
       <c r="D27" s="20" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E27" s="17" t="s">
         <v>57</v>
@@ -2847,16 +3175,16 @@
       </c>
       <c r="C28" s="16"/>
       <c r="D28" s="20" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E28" s="17" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="F28" s="17" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="G28" s="17" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="H28" s="17"/>
       <c r="I28" s="5"/>
@@ -2873,7 +3201,7 @@
       </c>
       <c r="C29" s="16"/>
       <c r="D29" s="20" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E29" s="17" t="s">
         <v>35</v>
@@ -2901,7 +3229,7 @@
         <v>4</v>
       </c>
       <c r="D30" s="20" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E30" s="17" t="s">
         <v>58</v>
@@ -2926,19 +3254,19 @@
         <v>18</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>63</v>
+        <v>3</v>
       </c>
       <c r="D31" s="20" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E31" s="19" t="s">
-        <v>233</v>
+        <v>326</v>
       </c>
       <c r="F31" s="19" t="s">
-        <v>233</v>
+        <v>326</v>
       </c>
       <c r="G31" s="19" t="s">
-        <v>233</v>
+        <v>326</v>
       </c>
       <c r="H31" s="5"/>
       <c r="I31" s="5"/>
@@ -2957,16 +3285,16 @@
         <v>63</v>
       </c>
       <c r="D32" s="20" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E32" s="19" t="s">
-        <v>234</v>
+        <v>328</v>
       </c>
       <c r="F32" s="19" t="s">
-        <v>234</v>
+        <v>328</v>
       </c>
       <c r="G32" s="19" t="s">
-        <v>234</v>
+        <v>328</v>
       </c>
       <c r="H32" s="5"/>
       <c r="I32" s="5"/>
@@ -2985,16 +3313,16 @@
         <v>4</v>
       </c>
       <c r="D33" s="20" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E33" s="17" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F33" s="17" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="G33" s="17" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="H33" s="5"/>
       <c r="I33" s="5"/>
@@ -3007,22 +3335,22 @@
         <v>92</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>20</v>
+        <v>327</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="D34" s="20" t="s">
-        <v>211</v>
-      </c>
-      <c r="E34" s="17" t="s">
-        <v>60</v>
-      </c>
-      <c r="F34" s="17" t="s">
-        <v>60</v>
-      </c>
-      <c r="G34" s="17" t="s">
-        <v>60</v>
+        <v>324</v>
+      </c>
+      <c r="E34" s="19" t="s">
+        <v>325</v>
+      </c>
+      <c r="F34" s="19" t="s">
+        <v>325</v>
+      </c>
+      <c r="G34" s="19" t="s">
+        <v>325</v>
       </c>
       <c r="H34" s="5"/>
       <c r="I34" s="5"/>
@@ -3035,22 +3363,22 @@
         <v>92</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>21</v>
+        <v>61</v>
       </c>
       <c r="C35" s="16" t="s">
-        <v>98</v>
+        <v>63</v>
       </c>
       <c r="D35" s="20" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E35" s="17" t="s">
-        <v>274</v>
+        <v>323</v>
       </c>
       <c r="F35" s="17" t="s">
-        <v>274</v>
+        <v>323</v>
       </c>
       <c r="G35" s="17" t="s">
-        <v>274</v>
+        <v>323</v>
       </c>
       <c r="H35" s="5"/>
       <c r="I35" s="5"/>
@@ -3063,22 +3391,22 @@
         <v>92</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="C36" s="16" t="s">
-        <v>186</v>
+        <v>63</v>
       </c>
       <c r="D36" s="20" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E36" s="17" t="s">
-        <v>277</v>
+        <v>64</v>
       </c>
       <c r="F36" s="17" t="s">
-        <v>277</v>
+        <v>64</v>
       </c>
       <c r="G36" s="17" t="s">
-        <v>277</v>
+        <v>64</v>
       </c>
       <c r="H36" s="5"/>
       <c r="I36" s="5"/>
@@ -3091,22 +3419,22 @@
         <v>92</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C37" s="16" t="s">
         <v>63</v>
       </c>
       <c r="D37" s="20" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E37" s="17" t="s">
-        <v>235</v>
+        <v>66</v>
       </c>
       <c r="F37" s="17" t="s">
-        <v>235</v>
+        <v>66</v>
       </c>
       <c r="G37" s="17" t="s">
-        <v>235</v>
+        <v>66</v>
       </c>
       <c r="H37" s="5"/>
       <c r="I37" s="5"/>
@@ -3119,22 +3447,22 @@
         <v>92</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>62</v>
+        <v>320</v>
       </c>
       <c r="C38" s="16" t="s">
         <v>63</v>
       </c>
       <c r="D38" s="20" t="s">
-        <v>215</v>
+        <v>321</v>
       </c>
       <c r="E38" s="17" t="s">
-        <v>64</v>
+        <v>322</v>
       </c>
       <c r="F38" s="17" t="s">
-        <v>64</v>
+        <v>322</v>
       </c>
       <c r="G38" s="17" t="s">
-        <v>64</v>
+        <v>322</v>
       </c>
       <c r="H38" s="5"/>
       <c r="I38" s="5"/>
@@ -3147,22 +3475,22 @@
         <v>92</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="C39" s="16" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D39" s="20" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="E39" s="17" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="F39" s="17" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="G39" s="17" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="H39" s="5"/>
       <c r="I39" s="5"/>
@@ -3175,50 +3503,50 @@
         <v>92</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>67</v>
+        <v>21</v>
       </c>
       <c r="C40" s="16" t="s">
-        <v>63</v>
+        <v>98</v>
       </c>
       <c r="D40" s="20" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="E40" s="17" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F40" s="17" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="G40" s="17" t="s">
-        <v>272</v>
-      </c>
-      <c r="H40" s="17"/>
+        <v>270</v>
+      </c>
+      <c r="H40" s="5"/>
       <c r="I40" s="5"/>
       <c r="J40" s="5"/>
       <c r="K40" s="5"/>
       <c r="L40" s="5"/>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A41" s="15" t="s">
-        <v>90</v>
+      <c r="A41" s="18" t="s">
+        <v>92</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>293</v>
+        <v>22</v>
       </c>
       <c r="C41" s="16" t="s">
-        <v>69</v>
+        <v>185</v>
       </c>
       <c r="D41" s="20" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="E41" s="17" t="s">
-        <v>70</v>
+        <v>273</v>
       </c>
       <c r="F41" s="17" t="s">
-        <v>70</v>
+        <v>273</v>
       </c>
       <c r="G41" s="17" t="s">
-        <v>70</v>
+        <v>273</v>
       </c>
       <c r="H41" s="5"/>
       <c r="I41" s="5"/>
@@ -3227,28 +3555,28 @@
       <c r="L41" s="5"/>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A42" s="15" t="s">
-        <v>90</v>
+      <c r="A42" s="18" t="s">
+        <v>92</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>181</v>
+        <v>67</v>
       </c>
       <c r="C42" s="16" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="D42" s="20" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="E42" s="17" t="s">
-        <v>72</v>
+        <v>268</v>
       </c>
       <c r="F42" s="17" t="s">
-        <v>72</v>
+        <v>268</v>
       </c>
       <c r="G42" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="H42" s="5"/>
+        <v>268</v>
+      </c>
+      <c r="H42" s="17"/>
       <c r="I42" s="5"/>
       <c r="J42" s="5"/>
       <c r="K42" s="5"/>
@@ -3259,22 +3587,22 @@
         <v>90</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="C43" s="16" t="s">
-        <v>4</v>
+        <v>69</v>
       </c>
       <c r="D43" s="20" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="E43" s="17" t="s">
-        <v>236</v>
-      </c>
-      <c r="F43" s="5" t="s">
-        <v>240</v>
-      </c>
-      <c r="G43" s="5" t="s">
-        <v>240</v>
+        <v>70</v>
+      </c>
+      <c r="F43" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="G43" s="17" t="s">
+        <v>70</v>
       </c>
       <c r="H43" s="5"/>
       <c r="I43" s="5"/>
@@ -3287,22 +3615,22 @@
         <v>90</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>74</v>
+        <v>181</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>4</v>
+        <v>71</v>
       </c>
       <c r="D44" s="20" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E44" s="17" t="s">
-        <v>237</v>
-      </c>
-      <c r="F44" s="5" t="s">
-        <v>241</v>
-      </c>
-      <c r="G44" s="5" t="s">
-        <v>241</v>
+        <v>72</v>
+      </c>
+      <c r="F44" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="G44" s="17" t="s">
+        <v>72</v>
       </c>
       <c r="H44" s="5"/>
       <c r="I44" s="5"/>
@@ -3315,22 +3643,22 @@
         <v>90</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>75</v>
+        <v>290</v>
       </c>
       <c r="C45" s="16" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D45" s="20" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="E45" s="17" t="s">
-        <v>76</v>
-      </c>
-      <c r="F45" s="17" t="s">
-        <v>76</v>
-      </c>
-      <c r="G45" s="17" t="s">
-        <v>76</v>
+        <v>232</v>
+      </c>
+      <c r="F45" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="G45" s="5" t="s">
+        <v>236</v>
       </c>
       <c r="H45" s="5"/>
       <c r="I45" s="5"/>
@@ -3343,22 +3671,22 @@
         <v>90</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C46" s="16" t="s">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="D46" s="20" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E46" s="17" t="s">
-        <v>78</v>
+        <v>233</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="G46" s="5" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="H46" s="5"/>
       <c r="I46" s="5"/>
@@ -3367,26 +3695,26 @@
       <c r="L46" s="5"/>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A47" s="18" t="s">
-        <v>91</v>
+      <c r="A47" s="15" t="s">
+        <v>90</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C47" s="16" t="s">
-        <v>69</v>
+        <v>1</v>
       </c>
       <c r="D47" s="20" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="E47" s="17" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F47" s="17" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="G47" s="17" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="H47" s="5"/>
       <c r="I47" s="5"/>
@@ -3395,26 +3723,26 @@
       <c r="L47" s="5"/>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A48" s="18" t="s">
-        <v>91</v>
+      <c r="A48" s="15" t="s">
+        <v>90</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C48" s="16" t="s">
-        <v>69</v>
+        <v>33</v>
       </c>
       <c r="D48" s="20" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="E48" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="F48" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="G48" s="17" t="s">
-        <v>82</v>
+        <v>78</v>
+      </c>
+      <c r="F48" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="G48" s="5" t="s">
+        <v>238</v>
       </c>
       <c r="H48" s="5"/>
       <c r="I48" s="5"/>
@@ -3427,22 +3755,22 @@
         <v>91</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C49" s="16" t="s">
-        <v>4</v>
+        <v>69</v>
       </c>
       <c r="D49" s="20" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="E49" s="17" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F49" s="17" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="G49" s="17" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="H49" s="5"/>
       <c r="I49" s="5"/>
@@ -3455,22 +3783,22 @@
         <v>91</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C50" s="16" t="s">
-        <v>4</v>
+        <v>69</v>
       </c>
       <c r="D50" s="20" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="E50" s="17" t="s">
-        <v>273</v>
+        <v>82</v>
       </c>
       <c r="F50" s="17" t="s">
-        <v>273</v>
+        <v>82</v>
       </c>
       <c r="G50" s="17" t="s">
-        <v>273</v>
+        <v>82</v>
       </c>
       <c r="H50" s="5"/>
       <c r="I50" s="5"/>
@@ -3479,26 +3807,26 @@
       <c r="L50" s="5"/>
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A51" s="15" t="s">
-        <v>111</v>
+      <c r="A51" s="18" t="s">
+        <v>91</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>182</v>
+        <v>83</v>
       </c>
       <c r="C51" s="16" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="D51" s="20" t="s">
-        <v>230</v>
-      </c>
-      <c r="E51" s="19" t="s">
-        <v>238</v>
-      </c>
-      <c r="F51" s="19" t="s">
-        <v>238</v>
-      </c>
-      <c r="G51" s="19" t="s">
-        <v>238</v>
+        <v>227</v>
+      </c>
+      <c r="E51" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="F51" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="G51" s="17" t="s">
+        <v>84</v>
       </c>
       <c r="H51" s="5"/>
       <c r="I51" s="5"/>
@@ -3507,26 +3835,26 @@
       <c r="L51" s="5"/>
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A52" s="15" t="s">
-        <v>111</v>
+      <c r="A52" s="18" t="s">
+        <v>91</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>183</v>
+        <v>85</v>
       </c>
       <c r="C52" s="16" t="s">
-        <v>71</v>
+        <v>4</v>
       </c>
       <c r="D52" s="20" t="s">
-        <v>231</v>
-      </c>
-      <c r="E52" s="19" t="s">
-        <v>239</v>
-      </c>
-      <c r="F52" s="19" t="s">
-        <v>239</v>
-      </c>
-      <c r="G52" s="19" t="s">
-        <v>239</v>
+        <v>228</v>
+      </c>
+      <c r="E52" s="17" t="s">
+        <v>269</v>
+      </c>
+      <c r="F52" s="17" t="s">
+        <v>269</v>
+      </c>
+      <c r="G52" s="17" t="s">
+        <v>269</v>
       </c>
       <c r="H52" s="5"/>
       <c r="I52" s="5"/>
@@ -3535,13 +3863,27 @@
       <c r="L52" s="5"/>
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A53" s="5"/>
-      <c r="B53" s="19"/>
-      <c r="C53" s="16"/>
-      <c r="D53" s="17"/>
-      <c r="E53" s="19"/>
-      <c r="F53" s="5"/>
-      <c r="G53" s="5"/>
+      <c r="A53" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="B53" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="C53" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="D53" s="20" t="s">
+        <v>229</v>
+      </c>
+      <c r="E53" s="19" t="s">
+        <v>234</v>
+      </c>
+      <c r="F53" s="19" t="s">
+        <v>234</v>
+      </c>
+      <c r="G53" s="19" t="s">
+        <v>234</v>
+      </c>
       <c r="H53" s="5"/>
       <c r="I53" s="5"/>
       <c r="J53" s="5"/>
@@ -3549,13 +3891,27 @@
       <c r="L53" s="5"/>
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A54" s="5"/>
-      <c r="B54" s="19"/>
-      <c r="C54" s="16"/>
-      <c r="D54" s="17"/>
-      <c r="E54" s="19"/>
-      <c r="F54" s="5"/>
-      <c r="G54" s="5"/>
+      <c r="A54" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="B54" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="C54" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="D54" s="20" t="s">
+        <v>230</v>
+      </c>
+      <c r="E54" s="19" t="s">
+        <v>235</v>
+      </c>
+      <c r="F54" s="19" t="s">
+        <v>235</v>
+      </c>
+      <c r="G54" s="19" t="s">
+        <v>235</v>
+      </c>
       <c r="H54" s="5"/>
       <c r="I54" s="5"/>
       <c r="J54" s="5"/>
@@ -4276,19 +4632,47 @@
       <c r="K105" s="5"/>
       <c r="L105" s="5"/>
     </row>
+    <row r="106" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A106" s="5"/>
+      <c r="B106" s="19"/>
+      <c r="C106" s="16"/>
+      <c r="D106" s="17"/>
+      <c r="E106" s="19"/>
+      <c r="F106" s="5"/>
+      <c r="G106" s="5"/>
+      <c r="H106" s="5"/>
+      <c r="I106" s="5"/>
+      <c r="J106" s="5"/>
+      <c r="K106" s="5"/>
+      <c r="L106" s="5"/>
+    </row>
+    <row r="107" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A107" s="5"/>
+      <c r="B107" s="19"/>
+      <c r="C107" s="16"/>
+      <c r="D107" s="17"/>
+      <c r="E107" s="19"/>
+      <c r="F107" s="5"/>
+      <c r="G107" s="5"/>
+      <c r="H107" s="5"/>
+      <c r="I107" s="5"/>
+      <c r="J107" s="5"/>
+      <c r="K107" s="5"/>
+      <c r="L107" s="5"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="B2:B7">
-    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2:B52">
-    <cfRule type="duplicateValues" dxfId="2" priority="5"/>
+  <conditionalFormatting sqref="B2:B54">
+    <cfRule type="duplicateValues" dxfId="3" priority="8"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B8:B52">
-    <cfRule type="duplicateValues" dxfId="1" priority="6"/>
+  <conditionalFormatting sqref="B8:B54">
+    <cfRule type="duplicateValues" dxfId="2" priority="10"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D52">
-    <cfRule type="duplicateValues" dxfId="0" priority="7"/>
+  <conditionalFormatting sqref="D2:D54">
+    <cfRule type="duplicateValues" dxfId="1" priority="12"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -4383,22 +4767,22 @@
         <v>95</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>3</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="H5" s="5"/>
       <c r="I5" s="5"/>
@@ -4414,7 +4798,7 @@
         <v>3</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>112</v>
@@ -4439,7 +4823,7 @@
         <v>4</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>159</v>
@@ -4464,7 +4848,7 @@
         <v>4</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>160</v>
@@ -4489,7 +4873,7 @@
         <v>114</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>164</v>
@@ -4514,7 +4898,7 @@
         <v>3</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>165</v>
@@ -4539,7 +4923,7 @@
         <v>71</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>166</v>
@@ -4564,7 +4948,7 @@
         <v>114</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>161</v>
@@ -4589,7 +4973,7 @@
         <v>3</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>162</v>
@@ -4614,7 +4998,7 @@
         <v>71</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>163</v>
@@ -4639,7 +5023,7 @@
         <v>114</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>161</v>
@@ -4664,7 +5048,7 @@
         <v>3</v>
       </c>
       <c r="D16" s="21" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>169</v>
@@ -4700,7 +5084,7 @@
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="21" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>145</v>
@@ -4732,20 +5116,20 @@
         <v>92</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="21" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="H20" s="5"/>
       <c r="I20" s="5"/>
@@ -4755,11 +5139,11 @@
         <v>92</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="C21" s="6"/>
       <c r="D21" s="21" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>146</v>
@@ -4781,19 +5165,19 @@
         <v>115</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="D22" s="21" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="H22" s="5"/>
       <c r="I22" s="5"/>
@@ -4809,7 +5193,7 @@
         <v>144</v>
       </c>
       <c r="D23" s="21" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>147</v>
@@ -4832,10 +5216,10 @@
       </c>
       <c r="C24" s="6"/>
       <c r="D24" s="21" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="F24" s="5" t="s">
         <v>125</v>
@@ -4857,7 +5241,7 @@
         <v>1</v>
       </c>
       <c r="D25" s="21" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="E25" s="5" t="s">
         <v>126</v>
@@ -4882,16 +5266,16 @@
         <v>124</v>
       </c>
       <c r="D26" s="21" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="H26" s="5"/>
       <c r="I26" s="5"/>
@@ -4907,7 +5291,7 @@
         <v>1</v>
       </c>
       <c r="D27" s="21" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="E27" s="5" t="s">
         <v>127</v>
@@ -4932,7 +5316,7 @@
         <v>69</v>
       </c>
       <c r="D28" s="21" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="E28" s="5" t="s">
         <v>136</v>
@@ -4957,7 +5341,7 @@
         <v>69</v>
       </c>
       <c r="D29" s="21" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="E29" s="5" t="s">
         <v>137</v>
@@ -4982,7 +5366,7 @@
         <v>1</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="E30" s="5" t="s">
         <v>138</v>
@@ -5007,7 +5391,7 @@
         <v>33</v>
       </c>
       <c r="D31" s="21" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="E31" s="5" t="s">
         <v>139</v>
@@ -5032,7 +5416,7 @@
         <v>69</v>
       </c>
       <c r="D32" s="21" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="E32" s="5" t="s">
         <v>140</v>
@@ -5057,7 +5441,7 @@
         <v>69</v>
       </c>
       <c r="D33" s="21" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="E33" s="5" t="s">
         <v>141</v>
@@ -5082,7 +5466,7 @@
         <v>1</v>
       </c>
       <c r="D34" s="21" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="E34" s="5" t="s">
         <v>142</v>
@@ -5105,7 +5489,7 @@
         <v>33</v>
       </c>
       <c r="D35" s="21" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="E35" s="5" t="s">
         <v>143</v>
@@ -5146,7 +5530,7 @@
         <v>4</v>
       </c>
       <c r="D1" s="21" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>148</v>
@@ -5171,7 +5555,7 @@
         <v>3</v>
       </c>
       <c r="D2" s="21" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>149</v>
@@ -5196,7 +5580,7 @@
         <v>114</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>150</v>

</xml_diff>

<commit_message>
Update eBus RCA model info workbook
</commit_message>
<xml_diff>
--- a/eBus_Functions/Post_Processing/Root_Cause_Analysis_Work/info/eBus_Model_Info.xlsx
+++ b/eBus_Functions/Post_Processing/Root_Cause_Analysis_Work/info/eBus_Model_Info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TempData\Github\eBus_Tool\eBus_Functions\Post_Processing\Root_Cause_Analysis_Work\info\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6579860E-F8BB-4EE3-915C-DF903BFDBA69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E79914EF-CCAB-49C9-9C0F-2D2CB603C8DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Block_Diagram" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="701" uniqueCount="332">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="727" uniqueCount="352">
   <si>
     <t>Driver</t>
   </si>
@@ -726,12 +726,6 @@
     <t>logout.pne_brk_Axle1_BrakingPower+logout.pne_brk_Axle2_BrakingPower+logout.pne_brk_Axle3_BrakingPower+logout.pne_brk_Axle4_BrakingPower</t>
   </si>
   <si>
-    <t>logout.eess_BatHW_P_BatPwr/1000</t>
-  </si>
-  <si>
-    <t>logout.eess_BatHW_P_BatLossPwr/1000</t>
-  </si>
-  <si>
     <t>logout.hvs_dcLink_aux_current</t>
   </si>
   <si>
@@ -1020,14 +1014,88 @@
     <t>Description</t>
   </si>
   <si>
-    <t>These Battery Current and Power Limits are sent to Powertrain Controller, so that power train controller can demand the torque, that is adhered to these limits</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In Vehicle Dynamics, 
+    <t>The Electric Drive System takes the Electric Motor Demand Torque from power train controller and gives out the actual electric motor torque, actual motor speed, actual motor electrical power, motor loss power. It also gives out the maximum and minimum  possible/available torque from electric drive system.</t>
+  </si>
+  <si>
+    <t>The sum of electric motor torques are input to Tranmission system. The transmission system can be of single speed or multi speed transmission. It gives out the Gear box torque, Gearbox speed, current Gear Number and Gear Ratio, Gearbox power loss</t>
+  </si>
+  <si>
+    <t>The gearbox output torque is fed to final drive. The output of final drive is the propulsion torque to wheel shaft.</t>
+  </si>
+  <si>
+    <t>The Pneumatic system, gives out the Friction Brake Force and Firction Brake Power</t>
+  </si>
+  <si>
+    <t>The Battery system caters the demand current. 
+The outputs from the Battery System are - Battery Current, Voltage, Power, Loss Power, State of Charge and Temperature</t>
+  </si>
+  <si>
+    <t>The Auxiliary Load System gives out the net auxiliary load current and voltage</t>
+  </si>
+  <si>
+    <t>Battery Charge Current Limit (Positive for Charge and Negative for Discharge)</t>
+  </si>
+  <si>
+    <t>Battery Discharge Current Limit (Positive for Charge and Negative for Discharge)</t>
+  </si>
+  <si>
+    <t>Battery Charge Power Limit (Positive for Charge and Negative for Discharge)</t>
+  </si>
+  <si>
+    <t>Battery Discharge Power Limit (Positive for Charge and Negative for Discharge)</t>
+  </si>
+  <si>
+    <t>The Driver model subsystem gets the Desired Velocity Input from Environmnet and Vehicle Velocity input from vehicle dynamics, the difference as an error is fed to PI (Proportional Integral) Controller. These driver model also has feedforward controller which makes use of the Vehicle Weight, Actual Gear Ration and Max Motor Torque information that assist in calculating the Acc Pedal and Brake Pedal along with PI controller. The accelerator and brake pedal are outcome of combination of PI and Feedforward controller.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Powertrain controller takes the Accelerator and Brake Pedal command from Driver model and demands the Electric Motor Torque from Electric drive system. 
+It gives out the Max and Min available electirc Motor demand torque.
+It also gives out the Max available Electric DrivingPower and Max available Electric Regeneration Power.
+The Powertrain controller also gets the information about Max Discharge Power and Max Charge Power from Battery Management System, State of Charge from Battery System. It also takes the feedback of Actual Motor Torque, Gear Ratio, Gear Number, Motor Torque-Speed profile data. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">In Vehicle Dynamics, the Force equations.
 Vehicle Propulsion Force = Net Traction Torque / Tire Radius;
-Vehicle Propulsion Force - Friction Brake Force = Wheel Force;
+Wheel Force = Vehicle Propulsion Force - Friction Brake Force;
 Wheel Force = AeroDynamic Force + Gradient Force + Rolling Resistance Force + Inertial Force;
+The inputs to the Vehicle Dynamics subsystems are the Vehicle Propulsion Force and Friction Brake Force.
+The outputs are Vehicle acceleration, velocity and distance. 
+It also gives out Aerodynamic Force, Gradient Force, Rolling Resistance Force and Intertial Force.
 </t>
+  </si>
+  <si>
+    <t>logout.eess_PresBatCur.*logout.eess_PresBatVolt/1000</t>
+  </si>
+  <si>
+    <t>logout.eess_BatHW_P_BatLossPwr.*sMP.phys.eess.BatHW_n_packs/1000</t>
+  </si>
+  <si>
+    <t>High Power Resistor</t>
+  </si>
+  <si>
+    <t>High Power Resistor Power</t>
+  </si>
+  <si>
+    <t>High Power Resistor Max allowed Power</t>
+  </si>
+  <si>
+    <t>hpr_pwr</t>
+  </si>
+  <si>
+    <t>hpr_max_pwr</t>
+  </si>
+  <si>
+    <t>logout.HPRS_Pwr_Cval</t>
+  </si>
+  <si>
+    <t>logout.HPRS_MaxPwr_Cval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Battery Management System calculates the Battery current limit and the power limit based on Ambient Temperature and State of Charge. These Battery Current and Power Limits are sent to Powertrain Controller, so that power train controller can demand the torque, that is adhered to these limits.
+Net Battery Power = Electric Motor 1 Power + Electric Motor 2 Power + Auxiliary Power + High Power Resistor Power </t>
+  </si>
+  <si>
+    <t>The High Power Resistor is activated during the regeneration braking on condition when power requirement for the auxiliary load and battery is fullfilled and left over power is dumped in HPR. The HPR is also activated, when there is heating requirment, which draws the power from battery.</t>
   </si>
 </sst>
 </file>
@@ -1370,26 +1438,12 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1408,27 +1462,59 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1503,22 +1589,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>485775</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:colOff>1524000</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>2972078</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>53340</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>4283317</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>17472</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
+        <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5FF86932-813C-2708-AD25-9E22B3903EE5}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{83846FB4-A9EC-5919-9D3A-5E3ED017C0C2}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1534,8 +1620,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1095375" y="771525"/>
-          <a:ext cx="9439553" cy="3444240"/>
+          <a:off x="2133600" y="238125"/>
+          <a:ext cx="10116427" cy="3774132"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1810,585 +1896,688 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="G27:J88"/>
+  <dimension ref="B27:H90"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="2" max="2" width="38.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="42.109375" style="41" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="121.44140625" style="12" customWidth="1"/>
     <col min="7" max="7" width="30.109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="26.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="54" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="82.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="27" spans="7:10" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="28" spans="7:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="G28" s="8" t="s">
+    <row r="27" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="28" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B28" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="H28" s="9" t="s">
+      <c r="C28" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="I28" s="10" t="s">
+      <c r="D28" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="J28" s="9" t="s">
+      <c r="E28" s="33" t="s">
+        <v>327</v>
+      </c>
+      <c r="H28"/>
+    </row>
+    <row r="29" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B29" s="22"/>
+      <c r="C29" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="D29" s="42" t="s">
+        <v>29</v>
+      </c>
+      <c r="E29" s="34"/>
+      <c r="H29"/>
+    </row>
+    <row r="30" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B30" s="23"/>
+      <c r="C30" s="28"/>
+      <c r="D30" s="43" t="s">
+        <v>7</v>
+      </c>
+      <c r="E30" s="35"/>
+      <c r="H30"/>
+    </row>
+    <row r="31" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B31" s="24"/>
+      <c r="C31" s="29"/>
+      <c r="D31" s="44" t="s">
+        <v>32</v>
+      </c>
+      <c r="E31" s="36"/>
+      <c r="H31"/>
+    </row>
+    <row r="32" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B32" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="C32" s="30" t="s">
+        <v>0</v>
+      </c>
+      <c r="D32" s="42" t="s">
+        <v>11</v>
+      </c>
+      <c r="E32" s="37" t="s">
+        <v>338</v>
+      </c>
+      <c r="H32"/>
+    </row>
+    <row r="33" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B33" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="C33" s="31"/>
+      <c r="D33" s="43" t="s">
+        <v>12</v>
+      </c>
+      <c r="E33" s="38"/>
+      <c r="H33"/>
+    </row>
+    <row r="34" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B34" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="C34" s="31"/>
+      <c r="D34" s="43"/>
+      <c r="E34" s="38"/>
+      <c r="H34"/>
+    </row>
+    <row r="35" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B35" s="23" t="s">
+        <v>13</v>
+      </c>
+      <c r="C35" s="31"/>
+      <c r="D35" s="43"/>
+      <c r="E35" s="38"/>
+      <c r="H35"/>
+    </row>
+    <row r="36" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B36" s="23" t="s">
+        <v>178</v>
+      </c>
+      <c r="C36" s="31"/>
+      <c r="D36" s="43"/>
+      <c r="E36" s="38"/>
+      <c r="H36"/>
+    </row>
+    <row r="37" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B37" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="C37" s="32"/>
+      <c r="D37" s="44"/>
+      <c r="E37" s="39"/>
+      <c r="H37"/>
+    </row>
+    <row r="38" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B38" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="C38" s="27" t="s">
+        <v>2</v>
+      </c>
+      <c r="D38" s="42" t="s">
+        <v>170</v>
+      </c>
+      <c r="E38" s="37" t="s">
+        <v>339</v>
+      </c>
+      <c r="H38"/>
+    </row>
+    <row r="39" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B39" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="C39" s="28"/>
+      <c r="D39" s="43" t="s">
+        <v>171</v>
+      </c>
+      <c r="E39" s="38"/>
+      <c r="H39"/>
+    </row>
+    <row r="40" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B40" s="23"/>
+      <c r="C40" s="28"/>
+      <c r="D40" s="43" t="s">
+        <v>300</v>
+      </c>
+      <c r="E40" s="38"/>
+      <c r="H40"/>
+    </row>
+    <row r="41" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B41" s="23"/>
+      <c r="C41" s="28"/>
+      <c r="D41" s="43" t="s">
+        <v>301</v>
+      </c>
+      <c r="E41" s="38"/>
+      <c r="H41"/>
+    </row>
+    <row r="42" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B42" s="23"/>
+      <c r="C42" s="28"/>
+      <c r="D42" s="43" t="s">
+        <v>304</v>
+      </c>
+      <c r="E42" s="38"/>
+      <c r="H42"/>
+    </row>
+    <row r="43" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B43" s="23"/>
+      <c r="C43" s="28"/>
+      <c r="D43" s="43" t="s">
+        <v>305</v>
+      </c>
+      <c r="E43" s="38"/>
+      <c r="H43"/>
+    </row>
+    <row r="44" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B44" s="23"/>
+      <c r="C44" s="28"/>
+      <c r="D44" s="43"/>
+      <c r="E44" s="38"/>
+      <c r="H44"/>
+    </row>
+    <row r="45" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B45" s="23"/>
+      <c r="C45" s="28"/>
+      <c r="D45" s="43"/>
+      <c r="E45" s="38"/>
+      <c r="H45"/>
+    </row>
+    <row r="46" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B46" s="23"/>
+      <c r="C46" s="28"/>
+      <c r="D46" s="43"/>
+      <c r="E46" s="38"/>
+      <c r="H46"/>
+    </row>
+    <row r="47" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B47" s="23"/>
+      <c r="C47" s="28"/>
+      <c r="D47" s="43"/>
+      <c r="E47" s="38"/>
+      <c r="H47"/>
+    </row>
+    <row r="48" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B48" s="24"/>
+      <c r="C48" s="29"/>
+      <c r="D48" s="44"/>
+      <c r="E48" s="39"/>
+      <c r="H48"/>
+    </row>
+    <row r="49" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B49" s="22" t="s">
+        <v>170</v>
+      </c>
+      <c r="C49" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="D49" s="45" t="s">
+        <v>36</v>
+      </c>
+      <c r="E49" s="37" t="s">
+        <v>328</v>
+      </c>
+      <c r="H49"/>
+    </row>
+    <row r="50" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B50" s="23" t="s">
+        <v>171</v>
+      </c>
+      <c r="C50" s="31"/>
+      <c r="D50" s="41" t="s">
+        <v>38</v>
+      </c>
+      <c r="E50" s="38"/>
+      <c r="H50"/>
+    </row>
+    <row r="51" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B51" s="23" t="s">
+        <v>302</v>
+      </c>
+      <c r="C51" s="31"/>
+      <c r="D51" s="41" t="s">
+        <v>40</v>
+      </c>
+      <c r="E51" s="38"/>
+      <c r="H51"/>
+    </row>
+    <row r="52" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B52" s="23" t="s">
+        <v>303</v>
+      </c>
+      <c r="C52" s="31"/>
+      <c r="D52" s="41" t="s">
+        <v>42</v>
+      </c>
+      <c r="E52" s="38"/>
+      <c r="H52"/>
+    </row>
+    <row r="53" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B53" s="23"/>
+      <c r="C53" s="31"/>
+      <c r="D53" s="41" t="s">
+        <v>44</v>
+      </c>
+      <c r="E53" s="38"/>
+      <c r="H53"/>
+    </row>
+    <row r="54" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B54" s="23"/>
+      <c r="C54" s="31"/>
+      <c r="D54" s="41" t="s">
+        <v>46</v>
+      </c>
+      <c r="E54" s="38"/>
+      <c r="H54"/>
+    </row>
+    <row r="55" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B55" s="23"/>
+      <c r="C55" s="31"/>
+      <c r="D55" s="41" t="s">
+        <v>172</v>
+      </c>
+      <c r="E55" s="38"/>
+      <c r="H55"/>
+    </row>
+    <row r="56" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B56" s="23"/>
+      <c r="C56" s="31"/>
+      <c r="D56" s="41" t="s">
+        <v>173</v>
+      </c>
+      <c r="E56" s="38"/>
+      <c r="H56"/>
+    </row>
+    <row r="57" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B57" s="23"/>
+      <c r="C57" s="31"/>
+      <c r="D57" s="41" t="s">
+        <v>50</v>
+      </c>
+      <c r="E57" s="38"/>
+      <c r="H57"/>
+    </row>
+    <row r="58" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B58" s="23"/>
+      <c r="C58" s="31"/>
+      <c r="D58" s="41" t="s">
+        <v>174</v>
+      </c>
+      <c r="E58" s="38"/>
+      <c r="H58"/>
+    </row>
+    <row r="59" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B59" s="23"/>
+      <c r="C59" s="31"/>
+      <c r="D59" s="41" t="s">
+        <v>53</v>
+      </c>
+      <c r="E59" s="38"/>
+      <c r="H59"/>
+    </row>
+    <row r="60" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B60" s="24"/>
+      <c r="C60" s="32"/>
+      <c r="D60" s="46" t="s">
+        <v>175</v>
+      </c>
+      <c r="E60" s="39"/>
+      <c r="H60"/>
+    </row>
+    <row r="61" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B61" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="C61" s="27" t="s">
+        <v>107</v>
+      </c>
+      <c r="D61" s="45" t="s">
+        <v>176</v>
+      </c>
+      <c r="E61" s="37" t="s">
         <v>329</v>
       </c>
-    </row>
-    <row r="29" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G29" s="22"/>
-      <c r="H29" s="37" t="s">
-        <v>6</v>
-      </c>
-      <c r="I29" s="23" t="s">
-        <v>29</v>
-      </c>
-      <c r="J29" s="28"/>
-    </row>
-    <row r="30" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G30" s="24"/>
-      <c r="H30" s="38"/>
-      <c r="I30" s="25" t="s">
-        <v>7</v>
-      </c>
-      <c r="J30" s="29"/>
-    </row>
-    <row r="31" spans="7:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="G31" s="26"/>
-      <c r="H31" s="39"/>
-      <c r="I31" s="27" t="s">
+      <c r="H61"/>
+    </row>
+    <row r="62" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B62" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="C62" s="28"/>
+      <c r="D62" s="41" t="s">
+        <v>177</v>
+      </c>
+      <c r="E62" s="38"/>
+      <c r="H62"/>
+    </row>
+    <row r="63" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B63" s="23"/>
+      <c r="C63" s="28"/>
+      <c r="D63" s="41" t="s">
+        <v>15</v>
+      </c>
+      <c r="E63" s="38"/>
+      <c r="H63"/>
+    </row>
+    <row r="64" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B64" s="23"/>
+      <c r="C64" s="28"/>
+      <c r="D64" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="E64" s="38"/>
+      <c r="H64"/>
+    </row>
+    <row r="65" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B65" s="24"/>
+      <c r="C65" s="29"/>
+      <c r="D65" s="46" t="s">
+        <v>16</v>
+      </c>
+      <c r="E65" s="39"/>
+      <c r="H65"/>
+    </row>
+    <row r="66" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B66" s="25" t="s">
+        <v>176</v>
+      </c>
+      <c r="C66" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="D66" s="47" t="s">
+        <v>18</v>
+      </c>
+      <c r="E66" s="40" t="s">
+        <v>330</v>
+      </c>
+      <c r="H66"/>
+    </row>
+    <row r="67" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B67" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="C67" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="D67" s="45" t="s">
+        <v>179</v>
+      </c>
+      <c r="E67" s="34" t="s">
+        <v>331</v>
+      </c>
+      <c r="H67"/>
+    </row>
+    <row r="68" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B68" s="24"/>
+      <c r="C68" s="32"/>
+      <c r="D68" s="46" t="s">
+        <v>180</v>
+      </c>
+      <c r="E68" s="36"/>
+      <c r="H68"/>
+    </row>
+    <row r="69" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B69" s="22" t="s">
+        <v>325</v>
+      </c>
+      <c r="C69" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="D69" s="45" t="s">
+        <v>20</v>
+      </c>
+      <c r="E69" s="37" t="s">
+        <v>340</v>
+      </c>
+      <c r="H69"/>
+    </row>
+    <row r="70" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B70" s="23" t="s">
+        <v>179</v>
+      </c>
+      <c r="C70" s="28"/>
+      <c r="D70" s="41" t="s">
+        <v>21</v>
+      </c>
+      <c r="E70" s="38"/>
+      <c r="H70"/>
+    </row>
+    <row r="71" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B71" s="23"/>
+      <c r="C71" s="28"/>
+      <c r="D71" s="41" t="s">
+        <v>22</v>
+      </c>
+      <c r="E71" s="38"/>
+      <c r="H71"/>
+    </row>
+    <row r="72" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B72" s="23"/>
+      <c r="C72" s="28"/>
+      <c r="D72" s="41" t="s">
+        <v>61</v>
+      </c>
+      <c r="E72" s="38"/>
+      <c r="H72"/>
+    </row>
+    <row r="73" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B73" s="23"/>
+      <c r="C73" s="28"/>
+      <c r="D73" s="41" t="s">
+        <v>62</v>
+      </c>
+      <c r="E73" s="38"/>
+      <c r="H73"/>
+    </row>
+    <row r="74" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B74" s="23"/>
+      <c r="C74" s="28"/>
+      <c r="D74" s="41" t="s">
+        <v>65</v>
+      </c>
+      <c r="E74" s="38"/>
+      <c r="H74"/>
+    </row>
+    <row r="75" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B75" s="23"/>
+      <c r="C75" s="28"/>
+      <c r="D75" s="41" t="s">
+        <v>318</v>
+      </c>
+      <c r="E75" s="38"/>
+      <c r="H75"/>
+    </row>
+    <row r="76" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B76" s="24"/>
+      <c r="C76" s="29"/>
+      <c r="D76" s="46" t="s">
+        <v>67</v>
+      </c>
+      <c r="E76" s="39"/>
+      <c r="H76"/>
+    </row>
+    <row r="77" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B77" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="J31" s="30"/>
-    </row>
-    <row r="32" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G32" s="22" t="s">
-        <v>21</v>
-      </c>
-      <c r="H32" s="40" t="s">
-        <v>0</v>
-      </c>
-      <c r="I32" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="J32" s="28"/>
-    </row>
-    <row r="33" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G33" s="24" t="s">
-        <v>29</v>
-      </c>
-      <c r="H33" s="41"/>
-      <c r="I33" s="25" t="s">
-        <v>12</v>
-      </c>
-      <c r="J33" s="29"/>
-    </row>
-    <row r="34" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G34" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="H34" s="41"/>
-      <c r="I34" s="25"/>
-      <c r="J34" s="29"/>
-    </row>
-    <row r="35" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G35" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="H35" s="41"/>
-      <c r="I35" s="25"/>
-      <c r="J35" s="29"/>
-    </row>
-    <row r="36" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G36" s="24" t="s">
-        <v>178</v>
-      </c>
-      <c r="H36" s="41"/>
-      <c r="I36" s="25"/>
-      <c r="J36" s="29"/>
-    </row>
-    <row r="37" spans="7:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="G37" s="26" t="s">
-        <v>14</v>
-      </c>
-      <c r="H37" s="42"/>
-      <c r="I37" s="27"/>
-      <c r="J37" s="30"/>
-    </row>
-    <row r="38" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G38" s="22" t="s">
-        <v>11</v>
-      </c>
-      <c r="H38" s="37" t="s">
-        <v>2</v>
-      </c>
-      <c r="I38" s="23" t="s">
-        <v>170</v>
-      </c>
-      <c r="J38" s="28"/>
-    </row>
-    <row r="39" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G39" s="24" t="s">
-        <v>12</v>
-      </c>
-      <c r="H39" s="38"/>
-      <c r="I39" s="25" t="s">
-        <v>171</v>
-      </c>
-      <c r="J39" s="29"/>
-    </row>
-    <row r="40" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G40" s="24"/>
-      <c r="H40" s="38"/>
-      <c r="I40" s="25" t="s">
-        <v>302</v>
-      </c>
-      <c r="J40" s="29"/>
-    </row>
-    <row r="41" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G41" s="24"/>
-      <c r="H41" s="38"/>
-      <c r="I41" s="25" t="s">
-        <v>303</v>
-      </c>
-      <c r="J41" s="29"/>
-    </row>
-    <row r="42" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G42" s="24"/>
-      <c r="H42" s="38"/>
-      <c r="I42" s="25" t="s">
-        <v>306</v>
-      </c>
-      <c r="J42" s="29"/>
-    </row>
-    <row r="43" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G43" s="24"/>
-      <c r="H43" s="38"/>
-      <c r="I43" s="25" t="s">
-        <v>307</v>
-      </c>
-      <c r="J43" s="29"/>
-    </row>
-    <row r="44" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G44" s="24"/>
-      <c r="H44" s="38"/>
-      <c r="I44" s="25"/>
-      <c r="J44" s="29"/>
-    </row>
-    <row r="45" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G45" s="24"/>
-      <c r="H45" s="38"/>
-      <c r="I45" s="25"/>
-      <c r="J45" s="29"/>
-    </row>
-    <row r="46" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G46" s="24"/>
-      <c r="H46" s="38"/>
-      <c r="I46" s="25"/>
-      <c r="J46" s="29"/>
-    </row>
-    <row r="47" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G47" s="24"/>
-      <c r="H47" s="38"/>
-      <c r="I47" s="25"/>
-      <c r="J47" s="29"/>
-    </row>
-    <row r="48" spans="7:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="G48" s="26"/>
-      <c r="H48" s="39"/>
-      <c r="I48" s="27"/>
-      <c r="J48" s="30"/>
-    </row>
-    <row r="49" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G49" s="22" t="s">
-        <v>170</v>
-      </c>
-      <c r="H49" s="40" t="s">
-        <v>106</v>
-      </c>
-      <c r="I49" s="31" t="s">
-        <v>36</v>
-      </c>
-      <c r="J49" s="28"/>
-    </row>
-    <row r="50" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G50" s="24" t="s">
-        <v>171</v>
-      </c>
-      <c r="H50" s="41"/>
-      <c r="I50" s="32" t="s">
-        <v>38</v>
-      </c>
-      <c r="J50" s="29"/>
-    </row>
-    <row r="51" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G51" s="24" t="s">
-        <v>304</v>
-      </c>
-      <c r="H51" s="41"/>
-      <c r="I51" s="32" t="s">
-        <v>40</v>
-      </c>
-      <c r="J51" s="29"/>
-    </row>
-    <row r="52" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G52" s="24" t="s">
-        <v>305</v>
-      </c>
-      <c r="H52" s="41"/>
-      <c r="I52" s="32" t="s">
-        <v>42</v>
-      </c>
-      <c r="J52" s="29"/>
-    </row>
-    <row r="53" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G53" s="24"/>
-      <c r="H53" s="41"/>
-      <c r="I53" s="32" t="s">
-        <v>44</v>
-      </c>
-      <c r="J53" s="29"/>
-    </row>
-    <row r="54" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G54" s="24"/>
-      <c r="H54" s="41"/>
-      <c r="I54" s="32" t="s">
-        <v>46</v>
-      </c>
-      <c r="J54" s="29"/>
-    </row>
-    <row r="55" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G55" s="24"/>
-      <c r="H55" s="41"/>
-      <c r="I55" s="32" t="s">
-        <v>172</v>
-      </c>
-      <c r="J55" s="29"/>
-    </row>
-    <row r="56" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G56" s="24"/>
-      <c r="H56" s="41"/>
-      <c r="I56" s="32" t="s">
-        <v>173</v>
-      </c>
-      <c r="J56" s="29"/>
-    </row>
-    <row r="57" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G57" s="24"/>
-      <c r="H57" s="41"/>
-      <c r="I57" s="32" t="s">
-        <v>50</v>
-      </c>
-      <c r="J57" s="29"/>
-    </row>
-    <row r="58" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G58" s="24"/>
-      <c r="H58" s="41"/>
-      <c r="I58" s="32" t="s">
-        <v>174</v>
-      </c>
-      <c r="J58" s="29"/>
-    </row>
-    <row r="59" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G59" s="24"/>
-      <c r="H59" s="41"/>
-      <c r="I59" s="32" t="s">
-        <v>53</v>
-      </c>
-      <c r="J59" s="29"/>
-    </row>
-    <row r="60" spans="7:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="G60" s="26"/>
-      <c r="H60" s="42"/>
-      <c r="I60" s="33" t="s">
-        <v>175</v>
-      </c>
-      <c r="J60" s="30"/>
-    </row>
-    <row r="61" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G61" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H61" s="37" t="s">
-        <v>107</v>
-      </c>
-      <c r="I61" s="31" t="s">
-        <v>176</v>
-      </c>
-      <c r="J61" s="28"/>
-    </row>
-    <row r="62" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G62" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="H62" s="38"/>
-      <c r="I62" s="32" t="s">
-        <v>177</v>
-      </c>
-      <c r="J62" s="29"/>
-    </row>
-    <row r="63" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G63" s="24"/>
-      <c r="H63" s="38"/>
-      <c r="I63" s="32" t="s">
-        <v>15</v>
-      </c>
-      <c r="J63" s="29"/>
-    </row>
-    <row r="64" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G64" s="24"/>
-      <c r="H64" s="38"/>
-      <c r="I64" s="32" t="s">
-        <v>178</v>
-      </c>
-      <c r="J64" s="29"/>
-    </row>
-    <row r="65" spans="7:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="G65" s="26"/>
-      <c r="H65" s="39"/>
-      <c r="I65" s="33" t="s">
-        <v>16</v>
-      </c>
-      <c r="J65" s="30"/>
-    </row>
-    <row r="66" spans="7:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="G66" s="34" t="s">
-        <v>176</v>
-      </c>
-      <c r="H66" s="43" t="s">
-        <v>17</v>
-      </c>
-      <c r="I66" s="35" t="s">
-        <v>18</v>
-      </c>
-      <c r="J66" s="36"/>
-    </row>
-    <row r="67" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G67" s="22" t="s">
-        <v>12</v>
-      </c>
-      <c r="H67" s="40" t="s">
-        <v>108</v>
-      </c>
-      <c r="I67" s="31" t="s">
-        <v>179</v>
-      </c>
-      <c r="J67" s="28"/>
-    </row>
-    <row r="68" spans="7:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="G68" s="26"/>
-      <c r="H68" s="42"/>
-      <c r="I68" s="33" t="s">
-        <v>180</v>
-      </c>
-      <c r="J68" s="30"/>
-    </row>
-    <row r="69" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G69" s="22" t="s">
-        <v>327</v>
-      </c>
-      <c r="H69" s="37" t="s">
-        <v>19</v>
-      </c>
-      <c r="I69" s="31" t="s">
-        <v>20</v>
-      </c>
-      <c r="J69" s="48" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="70" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G70" s="24" t="s">
-        <v>179</v>
-      </c>
-      <c r="H70" s="38"/>
-      <c r="I70" s="32" t="s">
-        <v>21</v>
-      </c>
-      <c r="J70" s="49"/>
-    </row>
-    <row r="71" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G71" s="24"/>
-      <c r="H71" s="38"/>
-      <c r="I71" s="32" t="s">
-        <v>22</v>
-      </c>
-      <c r="J71" s="49"/>
-    </row>
-    <row r="72" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G72" s="24"/>
-      <c r="H72" s="38"/>
-      <c r="I72" s="32" t="s">
-        <v>61</v>
-      </c>
-      <c r="J72" s="49"/>
-    </row>
-    <row r="73" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G73" s="24"/>
-      <c r="H73" s="38"/>
-      <c r="I73" s="32" t="s">
-        <v>62</v>
-      </c>
-      <c r="J73" s="49"/>
-    </row>
-    <row r="74" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G74" s="24"/>
-      <c r="H74" s="38"/>
-      <c r="I74" s="32" t="s">
-        <v>65</v>
-      </c>
-      <c r="J74" s="49"/>
-    </row>
-    <row r="75" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G75" s="24"/>
-      <c r="H75" s="38"/>
-      <c r="I75" s="44" t="s">
-        <v>320</v>
-      </c>
-      <c r="J75" s="49"/>
-    </row>
-    <row r="76" spans="7:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="G76" s="26"/>
-      <c r="H76" s="39"/>
-      <c r="I76" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="J76" s="50"/>
-    </row>
-    <row r="77" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G77" s="22" t="s">
+      <c r="C77" s="27" t="s">
+        <v>109</v>
+      </c>
+      <c r="D77" s="45" t="s">
+        <v>68</v>
+      </c>
+      <c r="E77" s="37" t="s">
+        <v>332</v>
+      </c>
+      <c r="H77"/>
+    </row>
+    <row r="78" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B78" s="23"/>
+      <c r="C78" s="28"/>
+      <c r="D78" s="41" t="s">
+        <v>181</v>
+      </c>
+      <c r="E78" s="38"/>
+      <c r="H78"/>
+    </row>
+    <row r="79" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B79" s="23"/>
+      <c r="C79" s="28"/>
+      <c r="D79" s="41" t="s">
+        <v>73</v>
+      </c>
+      <c r="E79" s="38"/>
+      <c r="H79"/>
+    </row>
+    <row r="80" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B80" s="23"/>
+      <c r="C80" s="28"/>
+      <c r="D80" s="41" t="s">
+        <v>74</v>
+      </c>
+      <c r="E80" s="38"/>
+      <c r="H80"/>
+    </row>
+    <row r="81" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B81" s="23"/>
+      <c r="C81" s="28"/>
+      <c r="D81" s="41" t="s">
+        <v>75</v>
+      </c>
+      <c r="E81" s="38"/>
+      <c r="H81"/>
+    </row>
+    <row r="82" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B82" s="24"/>
+      <c r="C82" s="29"/>
+      <c r="D82" s="46" t="s">
+        <v>77</v>
+      </c>
+      <c r="E82" s="39"/>
+      <c r="H82"/>
+    </row>
+    <row r="83" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B83" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="H77" s="37" t="s">
-        <v>109</v>
-      </c>
-      <c r="I77" s="31" t="s">
-        <v>68</v>
-      </c>
-      <c r="J77" s="45"/>
-    </row>
-    <row r="78" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G78" s="24"/>
-      <c r="H78" s="38"/>
-      <c r="I78" s="32" t="s">
-        <v>181</v>
-      </c>
-      <c r="J78" s="46"/>
-    </row>
-    <row r="79" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G79" s="24"/>
-      <c r="H79" s="38"/>
-      <c r="I79" s="32" t="s">
-        <v>73</v>
-      </c>
-      <c r="J79" s="46"/>
-    </row>
-    <row r="80" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G80" s="24"/>
-      <c r="H80" s="38"/>
-      <c r="I80" s="32" t="s">
-        <v>74</v>
-      </c>
-      <c r="J80" s="46"/>
-    </row>
-    <row r="81" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G81" s="24"/>
-      <c r="H81" s="38"/>
-      <c r="I81" s="32" t="s">
+      <c r="C83" s="30" t="s">
+        <v>110</v>
+      </c>
+      <c r="D83" s="45" t="s">
+        <v>79</v>
+      </c>
+      <c r="E83" s="37" t="s">
+        <v>350</v>
+      </c>
+      <c r="H83"/>
+    </row>
+    <row r="84" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B84" s="23" t="s">
         <v>75</v>
       </c>
-      <c r="J81" s="46"/>
-    </row>
-    <row r="82" spans="7:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="G82" s="26"/>
-      <c r="H82" s="39"/>
-      <c r="I82" s="33" t="s">
-        <v>77</v>
-      </c>
-      <c r="J82" s="47"/>
-    </row>
-    <row r="83" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G83" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="H83" s="40" t="s">
-        <v>110</v>
-      </c>
-      <c r="I83" s="31" t="s">
-        <v>79</v>
-      </c>
-      <c r="J83" s="48" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="84" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G84" s="24" t="s">
-        <v>75</v>
-      </c>
-      <c r="H84" s="41"/>
-      <c r="I84" s="32" t="s">
+      <c r="C84" s="31"/>
+      <c r="D84" s="41" t="s">
         <v>81</v>
       </c>
-      <c r="J84" s="49"/>
-    </row>
-    <row r="85" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G85" s="24"/>
-      <c r="H85" s="41"/>
-      <c r="I85" s="32" t="s">
+      <c r="E84" s="38"/>
+      <c r="H84"/>
+    </row>
+    <row r="85" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B85" s="23"/>
+      <c r="C85" s="31"/>
+      <c r="D85" s="41" t="s">
         <v>83</v>
       </c>
-      <c r="J85" s="49"/>
-    </row>
-    <row r="86" spans="7:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="G86" s="26"/>
-      <c r="H86" s="42"/>
-      <c r="I86" s="33" t="s">
+      <c r="E85" s="38"/>
+      <c r="H85"/>
+    </row>
+    <row r="86" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B86" s="24"/>
+      <c r="C86" s="32"/>
+      <c r="D86" s="46" t="s">
         <v>85</v>
       </c>
-      <c r="J86" s="50"/>
-    </row>
-    <row r="87" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G87" s="22"/>
-      <c r="H87" s="37" t="s">
+      <c r="E86" s="39"/>
+      <c r="H86"/>
+    </row>
+    <row r="87" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B87" s="22"/>
+      <c r="C87" s="27" t="s">
         <v>111</v>
       </c>
-      <c r="I87" s="31" t="s">
+      <c r="D87" s="45" t="s">
         <v>182</v>
       </c>
-      <c r="J87" s="28"/>
-    </row>
-    <row r="88" spans="7:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="G88" s="26"/>
-      <c r="H88" s="39"/>
-      <c r="I88" s="33" t="s">
+      <c r="E87" s="34" t="s">
+        <v>333</v>
+      </c>
+      <c r="H87"/>
+    </row>
+    <row r="88" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B88" s="23"/>
+      <c r="C88" s="28"/>
+      <c r="D88" s="48" t="s">
         <v>183</v>
       </c>
-      <c r="J88" s="30"/>
+      <c r="E88" s="35"/>
+      <c r="H88"/>
+    </row>
+    <row r="89" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B89" s="22"/>
+      <c r="C89" s="30" t="s">
+        <v>343</v>
+      </c>
+      <c r="D89" s="49" t="s">
+        <v>344</v>
+      </c>
+      <c r="E89" s="37" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="90" spans="2:8" ht="29.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B90" s="24"/>
+      <c r="C90" s="32"/>
+      <c r="D90" s="50" t="s">
+        <v>345</v>
+      </c>
+      <c r="E90" s="39"/>
     </row>
   </sheetData>
-  <mergeCells count="20">
-    <mergeCell ref="J87:J88"/>
-    <mergeCell ref="J77:J82"/>
-    <mergeCell ref="J69:J76"/>
-    <mergeCell ref="J67:J68"/>
-    <mergeCell ref="H38:H48"/>
-    <mergeCell ref="J83:J86"/>
-    <mergeCell ref="J29:J31"/>
-    <mergeCell ref="J32:J37"/>
-    <mergeCell ref="J38:J48"/>
-    <mergeCell ref="J49:J60"/>
-    <mergeCell ref="J61:J65"/>
-    <mergeCell ref="H77:H82"/>
-    <mergeCell ref="H83:H86"/>
-    <mergeCell ref="H61:H65"/>
-    <mergeCell ref="H69:H76"/>
-    <mergeCell ref="H87:H88"/>
-    <mergeCell ref="H29:H31"/>
-    <mergeCell ref="H32:H37"/>
-    <mergeCell ref="H49:H60"/>
-    <mergeCell ref="H67:H68"/>
+  <mergeCells count="22">
+    <mergeCell ref="C89:C90"/>
+    <mergeCell ref="E89:E90"/>
+    <mergeCell ref="C29:C31"/>
+    <mergeCell ref="C32:C37"/>
+    <mergeCell ref="C49:C60"/>
+    <mergeCell ref="C67:C68"/>
+    <mergeCell ref="E29:E31"/>
+    <mergeCell ref="E32:E37"/>
+    <mergeCell ref="E38:E48"/>
+    <mergeCell ref="E49:E60"/>
+    <mergeCell ref="E61:E65"/>
+    <mergeCell ref="E87:E88"/>
+    <mergeCell ref="E77:E82"/>
+    <mergeCell ref="E69:E76"/>
+    <mergeCell ref="E67:E68"/>
+    <mergeCell ref="C38:C48"/>
+    <mergeCell ref="E83:E86"/>
+    <mergeCell ref="C77:C82"/>
+    <mergeCell ref="C83:C86"/>
+    <mergeCell ref="C61:C65"/>
+    <mergeCell ref="C69:C76"/>
+    <mergeCell ref="C87:C88"/>
   </mergeCells>
-  <conditionalFormatting sqref="I29:I88 G29:G88">
-    <cfRule type="duplicateValues" dxfId="0" priority="13"/>
+  <conditionalFormatting sqref="B29:B88 D29:D90">
+    <cfRule type="duplicateValues" dxfId="4" priority="13"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2402,7 +2591,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="58.5546875" style="11" customWidth="1"/>
+    <col min="2" max="2" width="57" style="11" customWidth="1"/>
     <col min="3" max="3" width="19" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24.6640625" style="12" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="46.44140625" style="11" bestFit="1" customWidth="1"/>
@@ -2446,22 +2635,22 @@
         <v>96</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="C2" s="16" t="s">
+        <v>284</v>
+      </c>
+      <c r="D2" s="20" t="s">
         <v>285</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="E2" s="17" t="s">
         <v>286</v>
       </c>
-      <c r="D2" s="20" t="s">
-        <v>287</v>
-      </c>
-      <c r="E2" s="17" t="s">
-        <v>288</v>
-      </c>
       <c r="F2" s="17" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="H2" s="5"/>
       <c r="I2" s="5"/>
@@ -2564,13 +2753,13 @@
         <v>188</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
@@ -2592,13 +2781,13 @@
         <v>189</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="H7" s="5"/>
       <c r="I7" s="5"/>
@@ -2611,7 +2800,7 @@
         <v>97</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>3</v>
@@ -2639,7 +2828,7 @@
         <v>97</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C9" s="16" t="s">
         <v>3</v>
@@ -2667,22 +2856,22 @@
         <v>97</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C10" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="F10" s="17" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="H10" s="5"/>
       <c r="I10" s="5"/>
@@ -2695,22 +2884,22 @@
         <v>97</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C11" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="F11" s="17" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="G11" s="17" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="H11" s="5"/>
       <c r="I11" s="5"/>
@@ -2723,22 +2912,22 @@
         <v>97</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="C12" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="F12" s="17" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="G12" s="17" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="H12" s="5"/>
       <c r="I12" s="5"/>
@@ -2751,22 +2940,22 @@
         <v>97</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C13" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D13" s="20" t="s">
+        <v>313</v>
+      </c>
+      <c r="E13" s="17" t="s">
         <v>315</v>
       </c>
-      <c r="E13" s="17" t="s">
-        <v>317</v>
-      </c>
       <c r="F13" s="17" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="G13" s="17" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="H13" s="5"/>
       <c r="I13" s="5"/>
@@ -2779,7 +2968,7 @@
         <v>95</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>3</v>
@@ -2807,7 +2996,7 @@
         <v>95</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C15" s="16" t="s">
         <v>3</v>
@@ -2891,7 +3080,7 @@
         <v>95</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C18" s="16" t="s">
         <v>4</v>
@@ -2919,7 +3108,7 @@
         <v>95</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C19" s="16" t="s">
         <v>4</v>
@@ -3003,7 +3192,7 @@
         <v>95</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C22" s="16" t="s">
         <v>3</v>
@@ -3031,7 +3220,7 @@
         <v>95</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C23" s="16" t="s">
         <v>3</v>
@@ -3059,7 +3248,7 @@
         <v>95</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C24" s="16" t="s">
         <v>3</v>
@@ -3087,7 +3276,7 @@
         <v>95</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C25" s="16" t="s">
         <v>3</v>
@@ -3115,7 +3304,7 @@
         <v>94</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C26" s="16" t="s">
         <v>3</v>
@@ -3178,13 +3367,13 @@
         <v>206</v>
       </c>
       <c r="E28" s="17" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="F28" s="17" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="G28" s="17" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="H28" s="17"/>
       <c r="I28" s="5"/>
@@ -3260,13 +3449,13 @@
         <v>209</v>
       </c>
       <c r="E31" s="19" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="F31" s="19" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="G31" s="19" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="H31" s="5"/>
       <c r="I31" s="5"/>
@@ -3288,13 +3477,13 @@
         <v>217</v>
       </c>
       <c r="E32" s="19" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="F32" s="19" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="G32" s="19" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="H32" s="5"/>
       <c r="I32" s="5"/>
@@ -3335,22 +3524,22 @@
         <v>92</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C34" s="16" t="s">
         <v>63</v>
       </c>
       <c r="D34" s="20" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="E34" s="19" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="F34" s="19" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="G34" s="19" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="H34" s="5"/>
       <c r="I34" s="5"/>
@@ -3372,13 +3561,13 @@
         <v>213</v>
       </c>
       <c r="E35" s="17" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="F35" s="17" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="G35" s="17" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="H35" s="5"/>
       <c r="I35" s="5"/>
@@ -3447,22 +3636,22 @@
         <v>92</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C38" s="16" t="s">
         <v>63</v>
       </c>
       <c r="D38" s="20" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="E38" s="17" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="F38" s="17" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="G38" s="17" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="H38" s="5"/>
       <c r="I38" s="5"/>
@@ -3512,13 +3701,13 @@
         <v>211</v>
       </c>
       <c r="E40" s="17" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="F40" s="17" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="G40" s="17" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="H40" s="5"/>
       <c r="I40" s="5"/>
@@ -3540,13 +3729,13 @@
         <v>212</v>
       </c>
       <c r="E41" s="17" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="F41" s="17" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="G41" s="17" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="H41" s="5"/>
       <c r="I41" s="5"/>
@@ -3568,13 +3757,13 @@
         <v>216</v>
       </c>
       <c r="E42" s="17" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="F42" s="17" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="G42" s="17" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="H42" s="17"/>
       <c r="I42" s="5"/>
@@ -3587,7 +3776,7 @@
         <v>90</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C43" s="16" t="s">
         <v>69</v>
@@ -3643,7 +3832,7 @@
         <v>90</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C45" s="16" t="s">
         <v>4</v>
@@ -3652,13 +3841,13 @@
         <v>221</v>
       </c>
       <c r="E45" s="17" t="s">
-        <v>232</v>
+        <v>341</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="H45" s="5"/>
       <c r="I45" s="5"/>
@@ -3680,13 +3869,13 @@
         <v>222</v>
       </c>
       <c r="E46" s="17" t="s">
-        <v>233</v>
+        <v>342</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="G46" s="5" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="H46" s="5"/>
       <c r="I46" s="5"/>
@@ -3739,10 +3928,10 @@
         <v>78</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="G48" s="5" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="H48" s="5"/>
       <c r="I48" s="5"/>
@@ -3755,7 +3944,7 @@
         <v>91</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>79</v>
+        <v>334</v>
       </c>
       <c r="C49" s="16" t="s">
         <v>69</v>
@@ -3783,7 +3972,7 @@
         <v>91</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>81</v>
+        <v>335</v>
       </c>
       <c r="C50" s="16" t="s">
         <v>69</v>
@@ -3811,7 +4000,7 @@
         <v>91</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>83</v>
+        <v>336</v>
       </c>
       <c r="C51" s="16" t="s">
         <v>4</v>
@@ -3839,7 +4028,7 @@
         <v>91</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>85</v>
+        <v>337</v>
       </c>
       <c r="C52" s="16" t="s">
         <v>4</v>
@@ -3848,13 +4037,13 @@
         <v>228</v>
       </c>
       <c r="E52" s="17" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="F52" s="17" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="G52" s="17" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="H52" s="5"/>
       <c r="I52" s="5"/>
@@ -3876,13 +4065,13 @@
         <v>229</v>
       </c>
       <c r="E53" s="19" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="F53" s="19" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="G53" s="19" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="H53" s="5"/>
       <c r="I53" s="5"/>
@@ -3904,13 +4093,13 @@
         <v>230</v>
       </c>
       <c r="E54" s="19" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="F54" s="19" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="G54" s="19" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="H54" s="5"/>
       <c r="I54" s="5"/>
@@ -3919,13 +4108,27 @@
       <c r="L54" s="5"/>
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A55" s="5"/>
-      <c r="B55" s="19"/>
-      <c r="C55" s="16"/>
-      <c r="D55" s="17"/>
-      <c r="E55" s="19"/>
-      <c r="F55" s="5"/>
-      <c r="G55" s="5"/>
+      <c r="A55" s="18" t="s">
+        <v>343</v>
+      </c>
+      <c r="B55" s="19" t="s">
+        <v>344</v>
+      </c>
+      <c r="C55" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D55" s="20" t="s">
+        <v>346</v>
+      </c>
+      <c r="E55" s="19" t="s">
+        <v>348</v>
+      </c>
+      <c r="F55" s="19" t="s">
+        <v>348</v>
+      </c>
+      <c r="G55" s="19" t="s">
+        <v>348</v>
+      </c>
       <c r="H55" s="5"/>
       <c r="I55" s="5"/>
       <c r="J55" s="5"/>
@@ -3933,13 +4136,27 @@
       <c r="L55" s="5"/>
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A56" s="5"/>
-      <c r="B56" s="19"/>
-      <c r="C56" s="16"/>
-      <c r="D56" s="17"/>
-      <c r="E56" s="19"/>
-      <c r="F56" s="5"/>
-      <c r="G56" s="5"/>
+      <c r="A56" s="18" t="s">
+        <v>343</v>
+      </c>
+      <c r="B56" s="19" t="s">
+        <v>345</v>
+      </c>
+      <c r="C56" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="D56" s="20" t="s">
+        <v>347</v>
+      </c>
+      <c r="E56" s="19" t="s">
+        <v>349</v>
+      </c>
+      <c r="F56" s="19" t="s">
+        <v>349</v>
+      </c>
+      <c r="G56" s="19" t="s">
+        <v>349</v>
+      </c>
       <c r="H56" s="5"/>
       <c r="I56" s="5"/>
       <c r="J56" s="5"/>
@@ -4663,16 +4880,16 @@
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="B2:B7">
-    <cfRule type="duplicateValues" dxfId="4" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:B54">
-    <cfRule type="duplicateValues" dxfId="3" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8:B54">
-    <cfRule type="duplicateValues" dxfId="2" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="10"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D54">
-    <cfRule type="duplicateValues" dxfId="1" priority="12"/>
+  <conditionalFormatting sqref="D2:D56">
+    <cfRule type="duplicateValues" dxfId="0" priority="12"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -4686,7 +4903,7 @@
   <cols>
     <col min="1" max="1" width="29.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.6640625" style="1" customWidth="1"/>
     <col min="4" max="4" width="34.109375" customWidth="1"/>
     <col min="5" max="5" width="43.109375" customWidth="1"/>
     <col min="6" max="6" width="39" customWidth="1"/>
@@ -4767,22 +4984,22 @@
         <v>95</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>3</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="H5" s="5"/>
       <c r="I5" s="5"/>
@@ -4798,7 +5015,7 @@
         <v>3</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>112</v>
@@ -4823,7 +5040,7 @@
         <v>4</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>159</v>
@@ -4848,7 +5065,7 @@
         <v>4</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>160</v>
@@ -4873,7 +5090,7 @@
         <v>114</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>164</v>
@@ -4898,7 +5115,7 @@
         <v>3</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>165</v>
@@ -4923,7 +5140,7 @@
         <v>71</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>166</v>
@@ -4948,7 +5165,7 @@
         <v>114</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>161</v>
@@ -4973,7 +5190,7 @@
         <v>3</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>162</v>
@@ -4998,7 +5215,7 @@
         <v>71</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>163</v>
@@ -5023,7 +5240,7 @@
         <v>114</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>161</v>
@@ -5048,7 +5265,7 @@
         <v>3</v>
       </c>
       <c r="D16" s="21" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>169</v>
@@ -5084,7 +5301,7 @@
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="21" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>145</v>
@@ -5116,20 +5333,20 @@
         <v>92</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="21" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="H20" s="5"/>
       <c r="I20" s="5"/>
@@ -5139,11 +5356,11 @@
         <v>92</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="C21" s="6"/>
       <c r="D21" s="21" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>146</v>
@@ -5165,19 +5382,19 @@
         <v>115</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="D22" s="21" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="H22" s="5"/>
       <c r="I22" s="5"/>
@@ -5193,7 +5410,7 @@
         <v>144</v>
       </c>
       <c r="D23" s="21" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>147</v>
@@ -5216,10 +5433,10 @@
       </c>
       <c r="C24" s="6"/>
       <c r="D24" s="21" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="F24" s="5" t="s">
         <v>125</v>
@@ -5241,7 +5458,7 @@
         <v>1</v>
       </c>
       <c r="D25" s="21" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="E25" s="5" t="s">
         <v>126</v>
@@ -5266,16 +5483,16 @@
         <v>124</v>
       </c>
       <c r="D26" s="21" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="H26" s="5"/>
       <c r="I26" s="5"/>
@@ -5291,7 +5508,7 @@
         <v>1</v>
       </c>
       <c r="D27" s="21" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="E27" s="5" t="s">
         <v>127</v>
@@ -5316,7 +5533,7 @@
         <v>69</v>
       </c>
       <c r="D28" s="21" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="E28" s="5" t="s">
         <v>136</v>
@@ -5341,7 +5558,7 @@
         <v>69</v>
       </c>
       <c r="D29" s="21" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E29" s="5" t="s">
         <v>137</v>
@@ -5366,7 +5583,7 @@
         <v>1</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="E30" s="5" t="s">
         <v>138</v>
@@ -5391,7 +5608,7 @@
         <v>33</v>
       </c>
       <c r="D31" s="21" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="E31" s="5" t="s">
         <v>139</v>
@@ -5416,7 +5633,7 @@
         <v>69</v>
       </c>
       <c r="D32" s="21" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="E32" s="5" t="s">
         <v>140</v>
@@ -5441,7 +5658,7 @@
         <v>69</v>
       </c>
       <c r="D33" s="21" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="E33" s="5" t="s">
         <v>141</v>
@@ -5466,7 +5683,7 @@
         <v>1</v>
       </c>
       <c r="D34" s="21" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="E34" s="5" t="s">
         <v>142</v>
@@ -5489,7 +5706,7 @@
         <v>33</v>
       </c>
       <c r="D35" s="21" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="E35" s="5" t="s">
         <v>143</v>
@@ -5530,7 +5747,7 @@
         <v>4</v>
       </c>
       <c r="D1" s="21" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>148</v>
@@ -5555,7 +5772,7 @@
         <v>3</v>
       </c>
       <c r="D2" s="21" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>149</v>
@@ -5580,7 +5797,7 @@
         <v>114</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>150</v>

</xml_diff>